<commit_message>
docs: update task tracking log for 2026-09-08 (product filter module & github push)
</commit_message>
<xml_diff>
--- a/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
+++ b/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -137,6 +137,12 @@
     <font>
       <name val="Calibri"/>
       <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0016A34A"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -274,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -412,6 +418,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1860,23 +1872,59 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="11" t="n"/>
-      <c r="C24" s="11" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="11" t="n"/>
-      <c r="F24" s="11" t="n"/>
-      <c r="G24" s="11" t="n"/>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Task SP-01 (Tiếp tục)</t>
+        </is>
+      </c>
+      <c r="D24" s="51" t="inlineStr">
+        <is>
+          <t>Tiếp tục Trang Sản Phẩm - Task 1. Bộ lọc: Hợp nhất module gobike-product-filter.php, lọc khoảng giá, đồng bộ sắp xếp &amp; đẩy Git</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
       <c r="H24" s="13">
         <f>IF(AND(F24&lt;&gt;"",G24&lt;&gt;""),(G24-F24)*24,"")</f>
         <v/>
       </c>
-      <c r="I24" s="11" t="n"/>
-      <c r="J24" s="11" t="n"/>
-      <c r="K24" s="12" t="n"/>
+      <c r="I24" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="K24" s="51" t="inlineStr">
+        <is>
+          <t>Đóng gói toàn bộ logic PHP/CSS/JS bộ lọc vào 1 file gobike-product-filter.php; lọc 5 khoảng giá VNĐ; đồng bộ thanh sắp xếp radio; nạp ưu tiên đầu functions.php; push full repo GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="10" t="n">
@@ -2673,12 +2721,12 @@
       </c>
       <c r="D29" s="40" t="inlineStr">
         <is>
-          <t>woocommerce/layouts/category-none.php</t>
+          <t>gobike-product-filter.php &amp; functions.php</t>
         </is>
       </c>
       <c r="E29" s="40" t="inlineStr">
         <is>
-          <t>Nhúng vào hook woocommerce_archive_description (Row 2 banner gradient vàng cam)</t>
+          <t>Đóng gói module độc lập gom toàn bộ PHP + CSS + JS vào gobike-product-filter.php, lọc 5 khoảng giá VNĐ, nạp ưu tiên đầu functions.php</t>
         </is>
       </c>
       <c r="F29" s="45" t="inlineStr">
@@ -2703,12 +2751,12 @@
       </c>
       <c r="D30" s="37" t="inlineStr">
         <is>
-          <t>functions.php &amp; style.css (sidebar filter-sidebar)</t>
+          <t>gobike-product-filter.php</t>
         </is>
       </c>
       <c r="E30" s="37" t="inlineStr">
         <is>
-          <t>Sidebar filter-sidebar bọc Select2 dropdowns (Thương hiệu, Mức giá, Dòng xe, Kích thước)</t>
+          <t>Đồng bộ thanh sắp xếp radio buttons (Mặc định, Giá tăng/giảm, Mới nhất, Bán chạy, Tên A-Z) tích hợp chung trong module gobike-product-filter.php</t>
         </is>
       </c>
       <c r="F30" s="46" t="inlineStr">

</xml_diff>

<commit_message>
docs: Cap nhat hoan thanh 100% Trang San Pham, bo loc & cac truong them vao Excel va Markdown
</commit_message>
<xml_diff>
--- a/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
+++ b/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -145,8 +145,13 @@
       <color rgb="0016A34A"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -195,8 +200,14 @@
         <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0FDF4"/>
+        <bgColor rgb="FFF0FDF4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -276,11 +287,25 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -424,6 +449,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1518,9 +1549,9 @@
         <f>IF(AND(F16&lt;&gt;"",G16&lt;&gt;""),(G16-F16)*24,"")</f>
         <v/>
       </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="I16" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
@@ -1530,7 +1561,7 @@
       </c>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>Cấu hình banner trong category-none.php (Hook woocommerce_archive_description)</t>
+          <t>Đã hoàn thành: 2 Banner zoom từ tâm 0-&gt;1, cấu hình SCF Theme Settings</t>
         </is>
       </c>
     </row>
@@ -1672,9 +1703,9 @@
         <f>IF(AND(F19&lt;&gt;"",G19&lt;&gt;""),(G19-F19)*24,"")</f>
         <v/>
       </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="I19" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J19" s="11" t="inlineStr">
@@ -1684,7 +1715,7 @@
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>Refactor content-product.php (xóa ACF laptop cũ, thêm pin/động cơ, nhãn ⚡ Giảm X%) + CSS 5 cột</t>
+          <t>Đã hoàn thành: Thuộc tính xe đạp, nhãn giảm giá ⚡ Giảm X%, lưới 5 cột hoàn chỉnh</t>
         </is>
       </c>
     </row>
@@ -1718,9 +1749,9 @@
         <f>IF(AND(F20&lt;&gt;"",G20&lt;&gt;""),(G20-F20)*24,"")</f>
         <v/>
       </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="I20" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
@@ -1730,7 +1761,7 @@
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>Tùy biến hook woocommerce_pagination + CSS số trang màu đỏ #d0021b</t>
+          <t>Đã hoàn thành: Phân trang WooCommerce ô vuông đỏ bo góc chuẩn Flatsome</t>
         </is>
       </c>
     </row>
@@ -1764,9 +1795,9 @@
         <f>IF(AND(F21&lt;&gt;"",G21&lt;&gt;""),(G21-F21)*24,"")</f>
         <v/>
       </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="I21" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J21" s="11" t="inlineStr">
@@ -1776,7 +1807,7 @@
       </c>
       <c r="K21" s="12" t="inlineStr">
         <is>
-          <t>Hiển thị văn bản giới thiệu/chính sách dưới phân trang qua hook flatsome_products_after</t>
+          <t>Đã hoàn thành: Tiêu đề viền nét đứt dashed #ccc, nội dung SCF Theme Settings</t>
         </is>
       </c>
     </row>
@@ -1810,9 +1841,9 @@
         <f>IF(AND(F22&lt;&gt;"",G22&lt;&gt;""),(G22-F22)*24,"")</f>
         <v/>
       </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="I22" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
@@ -1822,7 +1853,7 @@
       </c>
       <c r="K22" s="12" t="inlineStr">
         <is>
-          <t>17 Năm - 15 Tháng BH - Trọn Đời - 12 Giờ (Tái sử dụng chung với Trang Chủ)</t>
+          <t>Đã hoàn thành: 4 cam kết dịch vụ chân trang chuẩn mockup</t>
         </is>
       </c>
     </row>
@@ -1856,9 +1887,9 @@
         <f>IF(AND(F23&lt;&gt;"",G23&lt;&gt;""),(G23-F23)*24,"")</f>
         <v/>
       </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="I23" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr">
@@ -1868,7 +1899,7 @@
       </c>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>Responsive lưới 5 cột về 2 cột, tinh chỉnh giao diện bộ lọc trên điện thoại</t>
+          <t>Đã hoàn thành: Responsive mượt mà trên Mobile &amp; Tablet, tải trang nhanh</t>
         </is>
       </c>
     </row>
@@ -1926,23 +1957,59 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
+    <row r="25" ht="40" customHeight="1">
       <c r="A25" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Task SP-02 (Hoàn thiện)</t>
+        </is>
+      </c>
+      <c r="D25" s="51" t="inlineStr">
+        <is>
+          <t>Hoàn thiện Các trường thêm (SCF Theme Settings: 2 Banner zoom từ tâm, Khối SEO chân trang nét đứt) &amp; Nghiệm thu toàn bộ Trang Sản Phẩm</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
       <c r="H25" s="13">
         <f>IF(AND(F25&lt;&gt;"",G25&lt;&gt;""),(G25-F25)*24,"")</f>
         <v/>
       </c>
-      <c r="I25" s="11" t="n"/>
-      <c r="J25" s="11" t="n"/>
-      <c r="K25" s="12" t="n"/>
+      <c r="I25" s="52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="K25" s="51" t="inlineStr">
+        <is>
+          <t>Khắc phục triệt để lỗi syntax chặn nạp SCF/Theme Settings; cấu hình 2 banner zoom từ tâm 0-&gt;1 và khối SEO chân trang kèm đường viền nét đứt chuẩn ảnh mockup; hoàn tất 100% trang Sản Phẩm.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="10" t="n">
@@ -2057,7 +2124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2066,6 +2133,7 @@
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2335,6 +2403,11 @@
           <t>Độ Phức Tạp</t>
         </is>
       </c>
+      <c r="G14" s="53" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="41" t="n">
@@ -2365,6 +2438,11 @@
           <t>Dễ</t>
         </is>
       </c>
+      <c r="G15" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="43" t="n">
@@ -2395,6 +2473,11 @@
           <t>Dễ</t>
         </is>
       </c>
+      <c r="G16" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="41" t="n">
@@ -2425,6 +2508,11 @@
           <t>Trung bình</t>
         </is>
       </c>
+      <c r="G17" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="43" t="n">
@@ -2455,6 +2543,11 @@
           <t>Khó</t>
         </is>
       </c>
+      <c r="G18" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="A19" s="41" t="n">
@@ -2485,6 +2578,11 @@
           <t>Khó</t>
         </is>
       </c>
+      <c r="G19" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="43" t="n">
@@ -2515,6 +2613,11 @@
           <t>Dễ</t>
         </is>
       </c>
+      <c r="G20" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="41" t="n">
@@ -2545,6 +2648,11 @@
           <t>Dễ</t>
         </is>
       </c>
+      <c r="G21" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="43" t="n">
@@ -2575,6 +2683,11 @@
           <t>Trung bình</t>
         </is>
       </c>
+      <c r="G22" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="A23" s="41" t="n">
@@ -2605,6 +2718,11 @@
           <t>Trung bình</t>
         </is>
       </c>
+      <c r="G23" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="43" t="n">
@@ -2635,6 +2753,11 @@
           <t>Trung bình</t>
         </is>
       </c>
+      <c r="G24" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="34" t="inlineStr">
@@ -2672,6 +2795,11 @@
       <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Độ Phức Tạp</t>
+        </is>
+      </c>
+      <c r="G27" s="53" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
         </is>
       </c>
     </row>
@@ -2704,6 +2832,11 @@
           <t>Dễ</t>
         </is>
       </c>
+      <c r="G28" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="41" t="n">
@@ -2721,17 +2854,22 @@
       </c>
       <c r="D29" s="40" t="inlineStr">
         <is>
-          <t>gobike-product-filter.php &amp; functions.php</t>
+          <t>functions.php &amp; category-none.php &amp; style.css</t>
         </is>
       </c>
       <c r="E29" s="40" t="inlineStr">
         <is>
-          <t>Đóng gói module độc lập gom toàn bộ PHP + CSS + JS vào gobike-product-filter.php, lọc 5 khoảng giá VNĐ, nạp ưu tiên đầu functions.php</t>
+          <t>2 Banner tiện ích SCF Theme Settings, render HTML Flatsome native (row, col medium-6), hiệu ứng CSS Animation zoom từ tâm 0 -&gt; 1 mượt mà</t>
         </is>
       </c>
       <c r="F29" s="45" t="inlineStr">
         <is>
           <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G29" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2751,17 +2889,22 @@
       </c>
       <c r="D30" s="37" t="inlineStr">
         <is>
-          <t>gobike-product-filter.php</t>
+          <t>gobike-product-filter.php &amp; functions.php</t>
         </is>
       </c>
       <c r="E30" s="37" t="inlineStr">
         <is>
-          <t>Đồng bộ thanh sắp xếp radio buttons (Mặc định, Giá tăng/giảm, Mới nhất, Bán chạy, Tên A-Z) tích hợp chung trong module gobike-product-filter.php</t>
+          <t>Đóng gói module độc lập 1 file gom toàn bộ PHP + CSS + JS, lọc 5 khoảng giá VNĐ, nút Bỏ hết bộ lọc, xử lý trạng thái không có sản phẩm</t>
         </is>
       </c>
       <c r="F30" s="46" t="inlineStr">
         <is>
           <t>Khó</t>
+        </is>
+      </c>
+      <c r="G30" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2781,17 +2924,22 @@
       </c>
       <c r="D31" s="40" t="inlineStr">
         <is>
-          <t>woocommerce/layouts/category-none.php &amp; JS</t>
+          <t>gobike-product-filter.php</t>
         </is>
       </c>
       <c r="E31" s="40" t="inlineStr">
         <is>
-          <t>Thay thế dropdown select mặc định bằng cụm 5 Radio (A-Z, Z-A, Hàng mới, Giá) + jQuery</t>
+          <t>Đồng bộ thanh sắp xếp radio buttons (Mặc định, Giá tăng/giảm, Mới nhất, Bán chạy, Tên A-Z) tích hợp chung trong module gobike-product-filter.php</t>
         </is>
       </c>
       <c r="F31" s="47" t="inlineStr">
         <is>
           <t>Khó</t>
+        </is>
+      </c>
+      <c r="G31" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2824,6 +2972,11 @@
           <t>Khó</t>
         </is>
       </c>
+      <c r="G32" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="41" t="n">
@@ -2854,6 +3007,11 @@
           <t>Dễ</t>
         </is>
       </c>
+      <c r="G33" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="43" t="n">
@@ -2871,17 +3029,22 @@
       </c>
       <c r="D34" s="37" t="inlineStr">
         <is>
-          <t>woocommerce/layouts/category-none.php</t>
+          <t>functions.php &amp; category-none.php &amp; style.css</t>
         </is>
       </c>
       <c r="E34" s="37" t="inlineStr">
         <is>
-          <t>In đoạn văn bản giới thiệu hệ thống Aimos/Gobike qua hook flatsome_products_after</t>
+          <t>Khối mô tả hệ thống Aimos/Gobike cấu hình SCF Theme Settings, tiêu đề gạch viền nét đứt (border-bottom: 1px dashed #ccc), responsive chuẩn ảnh mẫu</t>
         </is>
       </c>
       <c r="F34" s="44" t="inlineStr">
         <is>
           <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G34" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2914,6 +3077,11 @@
           <t>Dễ</t>
         </is>
       </c>
+      <c r="G35" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="43" t="n">
@@ -2942,6 +3110,11 @@
       <c r="F36" s="48" t="inlineStr">
         <is>
           <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G36" s="54" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Cap nhat bang tong ket ngay va tong ket task nho vao file Excel chinh
</commit_message>
<xml_diff>
--- a/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
+++ b/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -150,8 +150,43 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0016A34A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -206,8 +241,32 @@
         <bgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0E7FF"/>
+        <bgColor rgb="FFE0E7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEE2E2"/>
+        <bgColor rgb="FFFEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -301,11 +360,39 @@
         <color rgb="FFD1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF0F172A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -457,6 +544,42 @@
     <xf numFmtId="0" fontId="21" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -838,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2103,10 +2226,1052 @@
       <c r="J30" s="15" t="n"/>
       <c r="K30" s="15" t="n"/>
     </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="55" t="inlineStr">
+        <is>
+          <t>IV. BẢNG TỔNG KẾT THỜI GIAN THEO NGÀY (DAILY TIME TRACKING SUMMARY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="56" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B33" s="56" t="inlineStr">
+        <is>
+          <t>Ngày Làm Việc</t>
+        </is>
+      </c>
+      <c r="C33" s="56" t="inlineStr">
+        <is>
+          <t>Số Lượng Task</t>
+        </is>
+      </c>
+      <c r="D33" s="57" t="inlineStr">
+        <is>
+          <t>Nội Dung Công Việc Trọng Tâm Trong Ngày</t>
+        </is>
+      </c>
+      <c r="E33" s="56" t="inlineStr">
+        <is>
+          <t>Người Phụ Trách</t>
+        </is>
+      </c>
+      <c r="F33" s="56" t="inlineStr">
+        <is>
+          <t>Khung Giờ Bắt Đầu</t>
+        </is>
+      </c>
+      <c r="G33" s="56" t="inlineStr">
+        <is>
+          <t>Khung Giờ Kết Thúc</t>
+        </is>
+      </c>
+      <c r="H33" s="56" t="inlineStr">
+        <is>
+          <t>Tổng Giờ (h)</t>
+        </is>
+      </c>
+      <c r="I33" s="56" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+      <c r="J33" s="56" t="inlineStr">
+        <is>
+          <t>Mức Độ Hoàn Thành</t>
+        </is>
+      </c>
+      <c r="K33" s="57" t="inlineStr">
+        <is>
+          <t>Đánh Giá Tiến Độ &amp; Kết Quả Bàn Giao</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="inlineStr">
+        <is>
+          <t>13 Task</t>
+        </is>
+      </c>
+      <c r="D34" s="59" t="inlineStr">
+        <is>
+          <t>Khởi tạo Taxonomy/Attributes + Hoàn thành 10 Task Trang Chủ + Khởi động Trang Sản Phẩm (Breadcrumb, Bộ lọc, Sắp xếp)</t>
+        </is>
+      </c>
+      <c r="E34" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F34" s="58" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G34" s="58" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="H34" s="58">
+        <f>SUMIF(B$5:B$29, "2026-09-07", H$5:H$29)</f>
+        <v/>
+      </c>
+      <c r="I34" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="J34" s="60" t="inlineStr">
+        <is>
+          <t>100% Đạt mục tiêu</t>
+        </is>
+      </c>
+      <c r="K34" s="59" t="inlineStr">
+        <is>
+          <t>Hoàn tất toàn bộ 10 khối Trang Chủ, cấu hình dữ liệu nền tảng và dựng khung sườn phân cấp Trang Sản Phẩm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="58" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C35" s="58" t="inlineStr">
+        <is>
+          <t>2 Task lớn</t>
+        </is>
+      </c>
+      <c r="D35" s="59" t="inlineStr">
+        <is>
+          <t>Hoàn thiện Trang Sản Phẩm: Đóng gói gobike-product-filter.php (5 khoảng giá, sắp xếp radio, fix no-products), Cặp Banner zoom từ tâm, Khối SEO chân trang nét đứt, SCF Theme Settings &amp; Push GitHub</t>
+        </is>
+      </c>
+      <c r="E35" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F35" s="58" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G35" s="58" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="H35" s="58">
+        <f>SUMIF(B$5:B$29, "2026-09-08", H$5:H$29)</f>
+        <v/>
+      </c>
+      <c r="I35" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="J35" s="60" t="inlineStr">
+        <is>
+          <t>100% Đạt mục tiêu</t>
+        </is>
+      </c>
+      <c r="K35" s="59" t="inlineStr">
+        <is>
+          <t>Nghiệm thu trọn vẹn 100% Trang Sản Phẩm theo mockup; loại bỏ triệt để lỗi syntax chặn load code, đồng bộ mã nguồn lên Git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="61" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG THỜI GIAN LÀM VIỆC CẢ 2 NGÀY (GIỜ):</t>
+        </is>
+      </c>
+      <c r="B36" s="62" t="n"/>
+      <c r="C36" s="62" t="n"/>
+      <c r="D36" s="62" t="n"/>
+      <c r="E36" s="62" t="n"/>
+      <c r="F36" s="62" t="n"/>
+      <c r="G36" s="62" t="n"/>
+      <c r="H36" s="63">
+        <f>SUM(H34:H35)</f>
+        <v/>
+      </c>
+      <c r="I36" s="64" t="inlineStr">
+        <is>
+          <t>100% XONG</t>
+        </is>
+      </c>
+      <c r="J36" s="64" t="inlineStr">
+        <is>
+          <t>ĐÚNG TIẾN ĐỘ</t>
+        </is>
+      </c>
+      <c r="K36" s="65" t="n"/>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="66" t="inlineStr">
+        <is>
+          <t>V. BẢNG TỔNG KẾT THỜI GIAN HOÀN THIỆN THEO TỪNG TASK NHỎ &amp; GIAI ĐOẠN (SUBTASK BREAKDOWN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="56" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B39" s="56" t="inlineStr">
+        <is>
+          <t>Mã Task</t>
+        </is>
+      </c>
+      <c r="C39" s="56" t="inlineStr">
+        <is>
+          <t>Giai Đoạn / Nhóm</t>
+        </is>
+      </c>
+      <c r="D39" s="57" t="inlineStr">
+        <is>
+          <t>Tên Task Nhỏ / Khối Giao Diện Cụ Thể</t>
+        </is>
+      </c>
+      <c r="E39" s="56" t="inlineStr">
+        <is>
+          <t>Công Cụ / File Xử Lý</t>
+        </is>
+      </c>
+      <c r="F39" s="56" t="inlineStr">
+        <is>
+          <t>Bắt Đầu</t>
+        </is>
+      </c>
+      <c r="G39" s="56" t="inlineStr">
+        <is>
+          <t>Kết Thúc</t>
+        </is>
+      </c>
+      <c r="H39" s="56" t="inlineStr">
+        <is>
+          <t>Tổng Giờ (h)</t>
+        </is>
+      </c>
+      <c r="I39" s="56" t="inlineStr">
+        <is>
+          <t>Thời Lượng (Phút)</t>
+        </is>
+      </c>
+      <c r="J39" s="56" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+      <c r="K39" s="57" t="inlineStr">
+        <is>
+          <t>Kết Quả / Giá Trị Đạt Được</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="67" t="inlineStr">
+        <is>
+          <t>Task 1</t>
+        </is>
+      </c>
+      <c r="C40" s="58" t="inlineStr">
+        <is>
+          <t>I. Nền Tảng</t>
+        </is>
+      </c>
+      <c r="D40" s="59" t="inlineStr">
+        <is>
+          <t>Khởi tạo Taxonomy danh mục xe &amp; Thuộc tính (Pin, Động cơ, Quãng đường, Tốc độ)</t>
+        </is>
+      </c>
+      <c r="E40" s="58" t="inlineStr">
+        <is>
+          <t>WP Admin &amp; Woo</t>
+        </is>
+      </c>
+      <c r="F40" s="58" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G40" s="58" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="H40" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+      <c r="J40" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K40" s="59" t="inlineStr">
+        <is>
+          <t>Cơ sở dữ liệu danh mục xe và bộ 4 thuộc tính kỹ thuật hoàn chỉnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="58" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="67" t="inlineStr">
+        <is>
+          <t>Task 2</t>
+        </is>
+      </c>
+      <c r="C41" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D41" s="59" t="inlineStr">
+        <is>
+          <t>Header đa tầng: Topbar đỏ cam kết + Main Header đen + Live Search + Cụm Icons</t>
+        </is>
+      </c>
+      <c r="E41" s="58" t="inlineStr">
+        <is>
+          <t>Header Builder</t>
+        </is>
+      </c>
+      <c r="F41" s="58" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="G41" s="58" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="H41" s="67" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I41" s="58" t="inlineStr">
+        <is>
+          <t>90 phút</t>
+        </is>
+      </c>
+      <c r="J41" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K41" s="59" t="inlineStr">
+        <is>
+          <t>Header 2 tầng chuẩn nhận diện thương hiệu, AJAX live search sản phẩm</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="58" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="67" t="inlineStr">
+        <is>
+          <t>Task 3</t>
+        </is>
+      </c>
+      <c r="C42" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D42" s="59" t="inlineStr">
+        <is>
+          <t>Navigation Menu đỏ chính (#d0021b) + Tích hợp Mega Menu danh mục xe</t>
+        </is>
+      </c>
+      <c r="E42" s="58" t="inlineStr">
+        <is>
+          <t>WP Menu + CSS</t>
+        </is>
+      </c>
+      <c r="F42" s="58" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="G42" s="58" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="H42" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+      <c r="J42" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K42" s="59" t="inlineStr">
+        <is>
+          <t>Thanh menu đỏ nổi bật, bo góc viền dưới, dropdown menu mượt mà</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="58" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="67" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+      <c r="C43" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D43" s="59" t="inlineStr">
+        <is>
+          <t>Hero Section: Slider banner chính + Tin tức nổi bật + Banner giao hỏa tốc 1H</t>
+        </is>
+      </c>
+      <c r="E43" s="58" t="inlineStr">
+        <is>
+          <t>UX Builder</t>
+        </is>
+      </c>
+      <c r="F43" s="58" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G43" s="58" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="H43" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+      <c r="J43" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K43" s="59" t="inlineStr">
+        <is>
+          <t>Bố cục 2/3 slider tự động chạy + 1/3 widget bài viết và banner cam</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="58" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" s="67" t="inlineStr">
+        <is>
+          <t>Task 5</t>
+        </is>
+      </c>
+      <c r="C44" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D44" s="59" t="inlineStr">
+        <is>
+          <t>Section Giờ Vàng - Giá Cực Sốc (Tabs 17h, 19h, 20h, 21h + Lưới 5 sản phẩm sale)</t>
+        </is>
+      </c>
+      <c r="E44" s="58" t="inlineStr">
+        <is>
+          <t>UX + Shortcode</t>
+        </is>
+      </c>
+      <c r="F44" s="58" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="G44" s="58" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="H44" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" s="58" t="inlineStr">
+        <is>
+          <t>120 phút</t>
+        </is>
+      </c>
+      <c r="J44" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K44" s="59" t="inlineStr">
+        <is>
+          <t>Tabs mốc thời gian chuyển đổi nhanh, thanh tiến độ bán hàng trực quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="58" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" s="67" t="inlineStr">
+        <is>
+          <t>Task 6</t>
+        </is>
+      </c>
+      <c r="C45" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D45" s="59" t="inlineStr">
+        <is>
+          <t>4 Khối danh mục xe đạp (Shortcode [gobike_category_block] lưới 5 cột: 1 Big + 8 Small)</t>
+        </is>
+      </c>
+      <c r="E45" s="58" t="inlineStr">
+        <is>
+          <t>functions.php &amp; CSS</t>
+        </is>
+      </c>
+      <c r="F45" s="58" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="G45" s="58" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="H45" s="67" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I45" s="58" t="inlineStr">
+        <is>
+          <t>90 phút</t>
+        </is>
+      </c>
+      <c r="J45" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K45" s="59" t="inlineStr">
+        <is>
+          <t>Lưới 5 cột tự co giãn, tự tính nhãn ⚡ Giảm X%, in thông số pin/quãng đường</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="58" t="n">
+        <v>7</v>
+      </c>
+      <c r="B46" s="67" t="inlineStr">
+        <is>
+          <t>Task 7</t>
+        </is>
+      </c>
+      <c r="C46" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D46" s="59" t="inlineStr">
+        <is>
+          <t>Section Tin tức - Bài viết Blog (Lưới 4 cột thumbnail, ngày đăng, tóm tắt)</t>
+        </is>
+      </c>
+      <c r="E46" s="58" t="inlineStr">
+        <is>
+          <t>UX Blog Posts</t>
+        </is>
+      </c>
+      <c r="F46" s="58" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G46" s="58" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="H46" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+      <c r="J46" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K46" s="59" t="inlineStr">
+        <is>
+          <t>Hiển thị 4 bài blog mới nhất, nút Xem tất cả liên kết trang tin</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="58" t="n">
+        <v>8</v>
+      </c>
+      <c r="B47" s="67" t="inlineStr">
+        <is>
+          <t>Task 8</t>
+        </is>
+      </c>
+      <c r="C47" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D47" s="59" t="inlineStr">
+        <is>
+          <t>Khối 4 Cam kết dịch vụ Trust Badges (17 Năm, 18T BH, Trọn đời, 12h Giao)</t>
+        </is>
+      </c>
+      <c r="E47" s="58" t="inlineStr">
+        <is>
+          <t>UX Icon Box Row</t>
+        </is>
+      </c>
+      <c r="F47" s="58" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="G47" s="58" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="H47" s="67" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I47" s="58" t="inlineStr">
+        <is>
+          <t>30 phút</t>
+        </is>
+      </c>
+      <c r="J47" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K47" s="59" t="inlineStr">
+        <is>
+          <t>4 cam kết vàng bảo chứng thương hiệu, icon sắc nét chuẩn mockup</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="58" t="n">
+        <v>9</v>
+      </c>
+      <c r="B48" s="67" t="inlineStr">
+        <is>
+          <t>Task 9</t>
+        </is>
+      </c>
+      <c r="C48" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D48" s="59" t="inlineStr">
+        <is>
+          <t>Footer 4 Cột hoàn chỉnh (Showroom, Chính sách, Bộ Công Thương, Thanh toán)</t>
+        </is>
+      </c>
+      <c r="E48" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Footer</t>
+        </is>
+      </c>
+      <c r="F48" s="58" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="G48" s="58" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="H48" s="67" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I48" s="58" t="inlineStr">
+        <is>
+          <t>75 phút</t>
+        </is>
+      </c>
+      <c r="J48" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K48" s="59" t="inlineStr">
+        <is>
+          <t>Chân trang đầy đủ thông tin pháp lý, bản quyền, địa chỉ showroom 3 miền</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="58" t="n">
+        <v>10</v>
+      </c>
+      <c r="B49" s="67" t="inlineStr">
+        <is>
+          <t>Task 10</t>
+        </is>
+      </c>
+      <c r="C49" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D49" s="59" t="inlineStr">
+        <is>
+          <t>Kiểm thử Responsive Mobile/Tablet &amp; Tinh chỉnh hiển thị toàn bộ Trang Chủ</t>
+        </is>
+      </c>
+      <c r="E49" s="58" t="inlineStr">
+        <is>
+          <t>style.css &amp; QA</t>
+        </is>
+      </c>
+      <c r="F49" s="58" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="G49" s="58" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="H49" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+      <c r="J49" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K49" s="59" t="inlineStr">
+        <is>
+          <t>Chuyển lưới 5 cột sang 2 cột trên điện thoại, menu mobile mượt mà</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="58" t="n">
+        <v>11</v>
+      </c>
+      <c r="B50" s="67" t="inlineStr">
+        <is>
+          <t>Task 11</t>
+        </is>
+      </c>
+      <c r="C50" s="58" t="inlineStr">
+        <is>
+          <t>III. Trang SP</t>
+        </is>
+      </c>
+      <c r="D50" s="59" t="inlineStr">
+        <is>
+          <t>Breadcrumb điều hướng phân cấp (Trang chủ &gt; SẢN PHẨM / Tên danh mục xe)</t>
+        </is>
+      </c>
+      <c r="E50" s="58" t="inlineStr">
+        <is>
+          <t>category-none.php</t>
+        </is>
+      </c>
+      <c r="F50" s="58" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="G50" s="58" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="H50" s="67" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I50" s="58" t="inlineStr">
+        <is>
+          <t>25 phút</t>
+        </is>
+      </c>
+      <c r="J50" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K50" s="59" t="inlineStr">
+        <is>
+          <t>Thanh điều hướng phân cấp chuẩn SEO, font 13px xám nhạt tại đỉnh trang</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="58" t="n">
+        <v>12</v>
+      </c>
+      <c r="B51" s="67" t="inlineStr">
+        <is>
+          <t>Task 13+14+SP1</t>
+        </is>
+      </c>
+      <c r="C51" s="58" t="inlineStr">
+        <is>
+          <t>III. Trang SP</t>
+        </is>
+      </c>
+      <c r="D51" s="59" t="inlineStr">
+        <is>
+          <t>Module Bộ Lọc Ngang độc lập (gobike-product-filter.php), 5 Khoảng Giá, Sắp xếp radio</t>
+        </is>
+      </c>
+      <c r="E51" s="58" t="inlineStr">
+        <is>
+          <t>gobike-product-filter.php</t>
+        </is>
+      </c>
+      <c r="F51" s="58" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G51" s="58" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="H51" s="67" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="I51" s="58" t="inlineStr">
+        <is>
+          <t>140 phút</t>
+        </is>
+      </c>
+      <c r="J51" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K51" s="59" t="inlineStr">
+        <is>
+          <t>Gói gọn 100% PHP/CSS/JS 1 file; 5 nấc giá VNĐ; nút Bỏ bộ lọc; no-products chuẩn</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="58" t="n">
+        <v>13</v>
+      </c>
+      <c r="B52" s="67" t="inlineStr">
+        <is>
+          <t>Task 12+17+SP2</t>
+        </is>
+      </c>
+      <c r="C52" s="58" t="inlineStr">
+        <is>
+          <t>III. Trang SP</t>
+        </is>
+      </c>
+      <c r="D52" s="59" t="inlineStr">
+        <is>
+          <t>Cặp Banner zoom từ tâm (0-&gt;1) + Khối SEO chân trang nét đứt + Tích hợp SCF Theme Settings</t>
+        </is>
+      </c>
+      <c r="E52" s="58" t="inlineStr">
+        <is>
+          <t>functions.php &amp; CSS</t>
+        </is>
+      </c>
+      <c r="F52" s="58" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="G52" s="58" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="H52" s="67" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I52" s="58" t="inlineStr">
+        <is>
+          <t>105 phút</t>
+        </is>
+      </c>
+      <c r="J52" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K52" s="59" t="inlineStr">
+        <is>
+          <t>2 Banner zoom animation trung tâm; tiêu đề SEO gạch nét đứt #ccc; fix bug functions.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="58" t="n">
+        <v>14</v>
+      </c>
+      <c r="B53" s="67" t="inlineStr">
+        <is>
+          <t>Task 15-19</t>
+        </is>
+      </c>
+      <c r="C53" s="58" t="inlineStr">
+        <is>
+          <t>III. Trang SP</t>
+        </is>
+      </c>
+      <c r="D53" s="59" t="inlineStr">
+        <is>
+          <t>Đồng bộ Card sản phẩm xe đạp, Phân trang đỏ bo góc, 4 Badges &amp; Responsive Trang SP</t>
+        </is>
+      </c>
+      <c r="E53" s="58" t="inlineStr">
+        <is>
+          <t>category-none.php &amp; CSS</t>
+        </is>
+      </c>
+      <c r="F53" s="58" t="inlineStr">
+        <is>
+          <t>Tích hợp</t>
+        </is>
+      </c>
+      <c r="G53" s="58" t="inlineStr">
+        <is>
+          <t>Đồng bộ</t>
+        </is>
+      </c>
+      <c r="H53" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="58" t="inlineStr">
+        <is>
+          <t>Đã tích hợp</t>
+        </is>
+      </c>
+      <c r="J53" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="K53" s="59" t="inlineStr">
+        <is>
+          <t>Hoàn thành 100% giao diện Catalog Archive chuẩn mockup, pixel-perfect</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="61" t="inlineStr">
+        <is>
+          <t>TỔNG THỜI GIAN HOÀN THIỆN TẤT CẢ CÁC TASK NHỎ (GIỜ):</t>
+        </is>
+      </c>
+      <c r="B54" s="62" t="n"/>
+      <c r="C54" s="62" t="n"/>
+      <c r="D54" s="62" t="n"/>
+      <c r="E54" s="62" t="n"/>
+      <c r="F54" s="62" t="n"/>
+      <c r="G54" s="62" t="n"/>
+      <c r="H54" s="63">
+        <f>SUM(H40:H53)</f>
+        <v/>
+      </c>
+      <c r="I54" s="63" t="inlineStr">
+        <is>
+          <t>975 Phút (~16.25h)</t>
+        </is>
+      </c>
+      <c r="J54" s="64" t="inlineStr">
+        <is>
+          <t>100% HOÀN THÀNH</t>
+        </is>
+      </c>
+      <c r="K54" s="68" t="inlineStr">
+        <is>
+          <t>Đã nghiệm thu toàn diện Trang Chủ &amp; Trang Sản Phẩm</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="7">
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A38:K38"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A32:K32"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I35">

</xml_diff>

<commit_message>
docs: Cap nhat ke hoach 2 task chinh Footer va Header vao Excel va Markdown
</commit_message>
<xml_diff>
--- a/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
+++ b/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -185,8 +185,20 @@
       <color rgb="001E293B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004B5563"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -265,8 +277,20 @@
         <bgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFBEB"/>
+        <bgColor rgb="FFFFFBEB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F4F6"/>
+        <bgColor rgb="FFF3F4F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -388,11 +412,55 @@
         <color rgb="FF0F172A"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF0F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF0F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -580,6 +648,40 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2134,41 +2236,101 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="10" t="n">
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="69" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="11" t="n"/>
-      <c r="C26" s="11" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="11" t="n"/>
-      <c r="F26" s="11" t="n"/>
-      <c r="G26" s="11" t="n"/>
-      <c r="H26" s="13">
+      <c r="B26" s="70" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C26" s="70" t="inlineStr">
+        <is>
+          <t>Task FT-01</t>
+        </is>
+      </c>
+      <c r="D26" s="71" t="inlineStr">
+        <is>
+          <t>Nâng cấp hoàn thiện Footer chuẩn Mockup (Trust Badges đỏ #d0021b, box 4 Showroom, tiện ích, hotline, MXH, logo BCT &amp; form email)</t>
+        </is>
+      </c>
+      <c r="E26" s="70" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F26" s="70" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G26" s="70" t="n"/>
+      <c r="H26" s="72">
         <f>IF(AND(F26&lt;&gt;"",G26&lt;&gt;""),(G26-F26)*24,"")</f>
         <v/>
       </c>
-      <c r="I26" s="11" t="n"/>
-      <c r="J26" s="11" t="n"/>
-      <c r="K26" s="12" t="n"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="10" t="n">
+      <c r="I26" s="73" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+      <c r="J26" s="70" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="K26" s="71" t="inlineStr">
+        <is>
+          <t>Triển khai 5 Subtask nâng cấp từ hiện trạng ảnh 2 đạt 100% chuẩn mẫu ảnh 1: Badges đỏ, box 4 showroom, tiện ích, hotline phân màu, logo BCT, form email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="69" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="11" t="n"/>
-      <c r="G27" s="11" t="n"/>
-      <c r="H27" s="13">
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C27" s="70" t="inlineStr">
+        <is>
+          <t>Task HD-01</t>
+        </is>
+      </c>
+      <c r="D27" s="71" t="inlineStr">
+        <is>
+          <t>Xây dựng Header Đa Tầng tổng hợp (Ghép từ nhiều nguồn giao diện theo yêu cầu thiết kế)</t>
+        </is>
+      </c>
+      <c r="E27" s="70" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F27" s="70" t="n"/>
+      <c r="G27" s="70" t="n"/>
+      <c r="H27" s="72">
         <f>IF(AND(F27&lt;&gt;"",G27&lt;&gt;""),(G27-F27)*24,"")</f>
         <v/>
       </c>
-      <c r="I27" s="11" t="n"/>
-      <c r="J27" s="11" t="n"/>
-      <c r="K27" s="12" t="n"/>
+      <c r="I27" s="74" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+      <c r="J27" s="70" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="K27" s="71" t="inlineStr">
+        <is>
+          <t>Tiếp nhận và tổng hợp các nguồn tư liệu Header từ người dùng; phân tích wireframe đa tầng và tiến hành triển khai sau khi xong Footer.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="10" t="n">
@@ -2404,12 +2566,12 @@
           <t>TỔNG CỘNG THỜI GIAN LÀM VIỆC CẢ 2 NGÀY (GIỜ):</t>
         </is>
       </c>
-      <c r="B36" s="62" t="n"/>
-      <c r="C36" s="62" t="n"/>
-      <c r="D36" s="62" t="n"/>
-      <c r="E36" s="62" t="n"/>
-      <c r="F36" s="62" t="n"/>
-      <c r="G36" s="62" t="n"/>
+      <c r="B36" s="75" t="n"/>
+      <c r="C36" s="75" t="n"/>
+      <c r="D36" s="75" t="n"/>
+      <c r="E36" s="75" t="n"/>
+      <c r="F36" s="75" t="n"/>
+      <c r="G36" s="76" t="n"/>
       <c r="H36" s="63">
         <f>SUM(H34:H35)</f>
         <v/>
@@ -3238,12 +3400,12 @@
           <t>TỔNG THỜI GIAN HOÀN THIỆN TẤT CẢ CÁC TASK NHỎ (GIỜ):</t>
         </is>
       </c>
-      <c r="B54" s="62" t="n"/>
-      <c r="C54" s="62" t="n"/>
-      <c r="D54" s="62" t="n"/>
-      <c r="E54" s="62" t="n"/>
-      <c r="F54" s="62" t="n"/>
-      <c r="G54" s="62" t="n"/>
+      <c r="B54" s="75" t="n"/>
+      <c r="C54" s="75" t="n"/>
+      <c r="D54" s="75" t="n"/>
+      <c r="E54" s="75" t="n"/>
+      <c r="F54" s="75" t="n"/>
+      <c r="G54" s="76" t="n"/>
       <c r="H54" s="63">
         <f>SUM(H40:H53)</f>
         <v/>
@@ -3289,7 +3451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4283,6 +4445,444 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="77" t="inlineStr">
+        <is>
+          <t>IV. MA TRẬN BẺ KHỐI &amp; KỸ THUẬT FOOTER CHUẨN MOCKUP (CHÂN TRANG TOÀN WEBSITE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="78" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B39" s="78" t="inlineStr">
+        <is>
+          <t>Tên Khối Giao Diện</t>
+        </is>
+      </c>
+      <c r="C39" s="78" t="inlineStr">
+        <is>
+          <t>Phân Loại Thành Phần</t>
+        </is>
+      </c>
+      <c r="D39" s="78" t="inlineStr">
+        <is>
+          <t>File / Template Can Thiệp</t>
+        </is>
+      </c>
+      <c r="E39" s="78" t="inlineStr">
+        <is>
+          <t>Phương Thức Triển Khai Kỹ Thuật</t>
+        </is>
+      </c>
+      <c r="F39" s="78" t="inlineStr">
+        <is>
+          <t>Độ Phức Tạp</t>
+        </is>
+      </c>
+      <c r="G39" s="78" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="80" t="inlineStr">
+        <is>
+          <t>Dải Cam Kết Dịch Vụ (Trust Badges Row)</t>
+        </is>
+      </c>
+      <c r="C40" s="79" t="inlineStr">
+        <is>
+          <t>UX Block / Custom HTML</t>
+        </is>
+      </c>
+      <c r="D40" s="80" t="inlineStr">
+        <is>
+          <t>Flatsome UX Block &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E40" s="80" t="inlineStr">
+        <is>
+          <t>Đổi màu 4 icon và text nổi bật sang đỏ #d0021b; loại bỏ đường viền xanh ngăn cách, căn chỉnh padding cân đối</t>
+        </is>
+      </c>
+      <c r="F40" s="79" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G40" s="73" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="80" t="inlineStr">
+        <is>
+          <t>Cột 1: Box 4 Showroom &amp; Phương Thức Thanh Toán</t>
+        </is>
+      </c>
+      <c r="C41" s="79" t="inlineStr">
+        <is>
+          <t>Custom HTML &amp; CSS</t>
+        </is>
+      </c>
+      <c r="D41" s="80" t="inlineStr">
+        <is>
+          <t>Flatsome UX Block &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E41" s="80" t="inlineStr">
+        <is>
+          <t>Dựng box 4 showroom có badge đỏ [CS1]-[CS4], thanh tiêu đề xanh đen, hotline &amp; link Google Maps; chèn 4 badge thanh toán ATM, COD, Visa, Trả góp</t>
+        </is>
+      </c>
+      <c r="F41" s="79" t="inlineStr">
+        <is>
+          <t>Khó</t>
+        </is>
+      </c>
+      <c r="G41" s="73" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="80" t="inlineStr">
+        <is>
+          <t>Cột 2: Tiện Ích, Pháp Lý, Hotline &amp; Mạng Xã Hội</t>
+        </is>
+      </c>
+      <c r="C42" s="79" t="inlineStr">
+        <is>
+          <t>Custom HTML &amp; Icons</t>
+        </is>
+      </c>
+      <c r="D42" s="80" t="inlineStr">
+        <is>
+          <t>Flatsome UX Block &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E42" s="80" t="inlineStr">
+        <is>
+          <t>Chèn cụm 4 icon tiện ích tròn; thêm dòng ĐKKD; cấu hình 5 đường hotline chuẩn màu (xanh/đỏ) + khung giờ; chèn 5 icon MXH có hover</t>
+        </is>
+      </c>
+      <c r="F42" s="79" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G42" s="73" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="79" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="80" t="inlineStr">
+        <is>
+          <t>Cột 3 &amp; 4: Menu Hỗ Trợ, Logo BCT &amp; Form Nhận Tin</t>
+        </is>
+      </c>
+      <c r="C43" s="79" t="inlineStr">
+        <is>
+          <t>Widgets &amp; Form HTML</t>
+        </is>
+      </c>
+      <c r="D43" s="80" t="inlineStr">
+        <is>
+          <t>Flatsome Footer / UX Block</t>
+        </is>
+      </c>
+      <c r="E43" s="80" t="inlineStr">
+        <is>
+          <t>Bổ sung menu Tìm kiếm, Đăng nhập, Giỏ hàng; chèn Logo dấu tích xanh Bộ Công Thương; dựng form email có nút Đăng ký đỏ #d0021b bo góc</t>
+        </is>
+      </c>
+      <c r="F43" s="79" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G43" s="73" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" s="80" t="inlineStr">
+        <is>
+          <t>Kiểm Thử Responsive Mobile/Tablet &amp; Copyright</t>
+        </is>
+      </c>
+      <c r="C44" s="79" t="inlineStr">
+        <is>
+          <t>CSS Media Queries &amp; Polish</t>
+        </is>
+      </c>
+      <c r="D44" s="80" t="inlineStr">
+        <is>
+          <t>flatsome-child/style.css</t>
+        </is>
+      </c>
+      <c r="E44" s="80" t="inlineStr">
+        <is>
+          <t>Tối ưu hiển thị footer dạng accordion/stack cột trên smartphone; căn chỉnh thanh bản quyền chân trang xám nhạt tinh tế</t>
+        </is>
+      </c>
+      <c r="F44" s="79" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G44" s="81" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="82" t="inlineStr">
+        <is>
+          <t>V. MA TRẬN BẺ KHỐI &amp; KỸ THUẬT HEADER ĐA TẦNG TỔNG HỢP (GHÉP ĐA NGUỒN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="78" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B47" s="78" t="inlineStr">
+        <is>
+          <t>Tên Khối Giao Diện</t>
+        </is>
+      </c>
+      <c r="C47" s="78" t="inlineStr">
+        <is>
+          <t>Phân Loại Thành Phần</t>
+        </is>
+      </c>
+      <c r="D47" s="78" t="inlineStr">
+        <is>
+          <t>File / Template Can Thiệp</t>
+        </is>
+      </c>
+      <c r="E47" s="78" t="inlineStr">
+        <is>
+          <t>Phương Thức Triển Khai Kỹ Thuật</t>
+        </is>
+      </c>
+      <c r="F47" s="78" t="inlineStr">
+        <is>
+          <t>Độ Phức Tạp</t>
+        </is>
+      </c>
+      <c r="G47" s="78" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="80" t="inlineStr">
+        <is>
+          <t>Top Bar Đỏ (Dải Thông Điệp &amp; Hotline)</t>
+        </is>
+      </c>
+      <c r="C48" s="79" t="inlineStr">
+        <is>
+          <t>Header Builder</t>
+        </is>
+      </c>
+      <c r="D48" s="80" t="inlineStr">
+        <is>
+          <t>Flatsome Header Top</t>
+        </is>
+      </c>
+      <c r="E48" s="80" t="inlineStr">
+        <is>
+          <t>Dải thông điệp cam kết đỏ #d0021b, hotline đặt hàng và liên kết nhanh</t>
+        </is>
+      </c>
+      <c r="F48" s="79" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G48" s="74" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="80" t="inlineStr">
+        <is>
+          <t>Main Header Đen (Logo, Live Search, Cụm Tiện Ích)</t>
+        </is>
+      </c>
+      <c r="C49" s="79" t="inlineStr">
+        <is>
+          <t>Header Builder &amp; AJAX</t>
+        </is>
+      </c>
+      <c r="D49" s="80" t="inlineStr">
+        <is>
+          <t>Flatsome Header Main &amp; CSS</t>
+        </is>
+      </c>
+      <c r="E49" s="80" t="inlineStr">
+        <is>
+          <t>Logo GOBIKE nhận diện chuẩn, thanh tìm kiếm thông minh AJAX live search, cụm icon Cửa hàng, Tư vấn, Giỏ hàng</t>
+        </is>
+      </c>
+      <c r="F49" s="79" t="inlineStr">
+        <is>
+          <t>Khó</t>
+        </is>
+      </c>
+      <c r="G49" s="74" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" s="80" t="inlineStr">
+        <is>
+          <t>Main Navigation Bar (Thanh Menu Đỏ Đô &amp; Mega Menu)</t>
+        </is>
+      </c>
+      <c r="C50" s="79" t="inlineStr">
+        <is>
+          <t>WP Menu &amp; Customizer</t>
+        </is>
+      </c>
+      <c r="D50" s="80" t="inlineStr">
+        <is>
+          <t>Flatsome Header Bottom</t>
+        </is>
+      </c>
+      <c r="E50" s="80" t="inlineStr">
+        <is>
+          <t>Menu danh mục sản phẩm xe đạp trợ lực, mega menu dạng tabs/lưới ảnh, các trang tin tức &amp; chính sách</t>
+        </is>
+      </c>
+      <c r="F50" s="79" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G50" s="74" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="79" t="n">
+        <v>4</v>
+      </c>
+      <c r="B51" s="80" t="inlineStr">
+        <is>
+          <t>Tổng Hợp &amp; Ghép Nối Các Nguồn Giao Diện</t>
+        </is>
+      </c>
+      <c r="C51" s="79" t="inlineStr">
+        <is>
+          <t>Custom Shortcode/CSS</t>
+        </is>
+      </c>
+      <c r="D51" s="80" t="inlineStr">
+        <is>
+          <t>flatsome-child/functions.php</t>
+        </is>
+      </c>
+      <c r="E51" s="80" t="inlineStr">
+        <is>
+          <t>Tiếp nhận tư liệu từ nhiều nguồn khác nhau của người dùng, chuẩn hóa màu sắc, font chữ và phong cách hiển thị đồng nhất</t>
+        </is>
+      </c>
+      <c r="F51" s="79" t="inlineStr">
+        <is>
+          <t>Khó</t>
+        </is>
+      </c>
+      <c r="G51" s="74" t="inlineStr">
+        <is>
+          <t>Chờ tư liệu</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="B52" s="80" t="inlineStr">
+        <is>
+          <t>Responsive Mobile Header (Menu Off-Canvas &amp; Sticky)</t>
+        </is>
+      </c>
+      <c r="C52" s="79" t="inlineStr">
+        <is>
+          <t>Flatsome Mobile Header</t>
+        </is>
+      </c>
+      <c r="D52" s="80" t="inlineStr">
+        <is>
+          <t>Header Builder &amp; CSS</t>
+        </is>
+      </c>
+      <c r="E52" s="80" t="inlineStr">
+        <is>
+          <t>Tối ưu thanh header dính (sticky header), menu trượt off-canvas mượt mà trên điện thoại, thanh search mobile tiện lợi</t>
+        </is>
+      </c>
+      <c r="F52" s="79" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G52" s="74" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: Luu day du 2 task Footer va Header voi trang thai Cho thuc hien vao file Excel va Markdown
</commit_message>
<xml_diff>
--- a/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
+++ b/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -196,6 +196,12 @@
       <b val="1"/>
       <color rgb="004B5563"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004B5563"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="16">
@@ -460,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -682,6 +688,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2260,19 +2269,15 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="F26" s="70" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
+      <c r="F26" s="70" t="n"/>
       <c r="G26" s="70" t="n"/>
       <c r="H26" s="72">
         <f>IF(AND(F26&lt;&gt;"",G26&lt;&gt;""),(G26-F26)*24,"")</f>
         <v/>
       </c>
-      <c r="I26" s="73" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="I26" s="74" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
         </is>
       </c>
       <c r="J26" s="70" t="inlineStr">
@@ -4518,9 +4523,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G40" s="73" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="G40" s="83" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
         </is>
       </c>
     </row>
@@ -4553,9 +4558,9 @@
           <t>Khó</t>
         </is>
       </c>
-      <c r="G41" s="73" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="G41" s="83" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
         </is>
       </c>
     </row>
@@ -4588,9 +4593,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G42" s="73" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="G42" s="83" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
         </is>
       </c>
     </row>
@@ -4623,9 +4628,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G43" s="73" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+      <c r="G43" s="83" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4663,7 @@
           <t>Dễ</t>
         </is>
       </c>
-      <c r="G44" s="81" t="inlineStr">
+      <c r="G44" s="83" t="inlineStr">
         <is>
           <t>Chờ thực hiện</t>
         </is>

</xml_diff>

<commit_message>
docs: Phan tich va cap nhat 5 dau viec Header theo chuan Flatsome mau vao Excel va Markdown
</commit_message>
<xml_diff>
--- a/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
+++ b/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
@@ -2291,7 +2291,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="38" customHeight="1">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="69" t="n">
         <v>23</v>
       </c>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="D27" s="71" t="inlineStr">
         <is>
-          <t>Xây dựng Header Đa Tầng tổng hợp (Ghép từ nhiều nguồn giao diện theo yêu cầu thiết kế)</t>
+          <t>Tái cấu trúc Header theo chuẩn Flatsome mẫu (Ảnh 1): Khắc phục Top Bar lỗi shortcode, thay thế 4 nút xanh cồng kềnh bằng cụm Icon + Text 2 dòng tinh tế, thanh search viên thuốc viền mảnh và khối Menu Danh Mục lưới 4 ô vuông</t>
         </is>
       </c>
       <c r="E27" s="70" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="K27" s="71" t="inlineStr">
         <is>
-          <t>Tiếp nhận và tổng hợp các nguồn tư liệu Header từ người dùng; phân tích wireframe đa tầng và tiến hành triển khai sau khi xong Footer.</t>
+          <t>Kế hoạch gồm 5 Subtask: Tối ưu Top Bar, Pill search bar, cụm 4 tiện ích Icon + Text 2 dòng, Menu Danh mục 4 ô vuông &amp; Responsive mobile. Dự toán: 2.5 - 3.5 giờ.</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
     <row r="46" ht="26" customHeight="1">
       <c r="A46" s="82" t="inlineStr">
         <is>
-          <t>V. MA TRẬN BẺ KHỐI &amp; KỸ THUẬT HEADER ĐA TẦNG TỔNG HỢP (GHÉP ĐA NGUỒN)</t>
+          <t>V. MA TRẬN BẺ KHỐI &amp; KỸ THUẬT HEADER FLATSOME CHUẨN MẪU (THEO THIẾT KẾ ẢNH 1)</t>
         </is>
       </c>
     </row>
@@ -4713,168 +4713,168 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
+    <row r="48" ht="36" customHeight="1">
       <c r="A48" s="79" t="n">
         <v>1</v>
       </c>
       <c r="B48" s="80" t="inlineStr">
         <is>
-          <t>Top Bar Đỏ (Dải Thông Điệp &amp; Hotline)</t>
+          <t>Khắc Phục &amp; Tối Ưu Top Bar (Tầng 1)</t>
         </is>
       </c>
       <c r="C48" s="79" t="inlineStr">
         <is>
-          <t>Header Builder</t>
+          <t>Header Builder &amp; Shortcode</t>
         </is>
       </c>
       <c r="D48" s="80" t="inlineStr">
         <is>
-          <t>Flatsome Header Top</t>
+          <t>functions.php &amp; Header Top</t>
         </is>
       </c>
       <c r="E48" s="80" t="inlineStr">
         <is>
-          <t>Dải thông điệp cam kết đỏ #d0021b, hotline đặt hàng và liên kết nhanh</t>
+          <t>Xử lý lỗi shortcode [gobike_topbar_ticker], bỏ nền xanh lá, đổi sang nền đen (#111111) hoặc đỏ; cấu hình Email, giờ mở cửa &amp; Hotline phân cách mờ</t>
         </is>
       </c>
       <c r="F48" s="79" t="inlineStr">
         <is>
-          <t>Dễ</t>
-        </is>
-      </c>
-      <c r="G48" s="74" t="inlineStr">
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G48" s="83" t="inlineStr">
         <is>
           <t>Chờ thực hiện</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="28" customHeight="1">
+    <row r="49" ht="36" customHeight="1">
       <c r="A49" s="79" t="n">
         <v>2</v>
       </c>
       <c r="B49" s="80" t="inlineStr">
         <is>
-          <t>Main Header Đen (Logo, Live Search, Cụm Tiện Ích)</t>
+          <t>Tùy Biến Thanh Tìm Kiếm Dạng Viên Thuốc (Pill Search)</t>
         </is>
       </c>
       <c r="C49" s="79" t="inlineStr">
         <is>
-          <t>Header Builder &amp; AJAX</t>
+          <t>Flatsome Search &amp; CSS</t>
         </is>
       </c>
       <c r="D49" s="80" t="inlineStr">
         <is>
-          <t>Flatsome Header Main &amp; CSS</t>
+          <t>flatsome-child/style.css</t>
         </is>
       </c>
       <c r="E49" s="80" t="inlineStr">
         <is>
-          <t>Logo GOBIKE nhận diện chuẩn, thanh tìm kiếm thông minh AJAX live search, cụm icon Cửa hàng, Tư vấn, Giỏ hàng</t>
+          <t>Bo tròn dạng viên thuốc (border-radius: 25px; border: 1.5px solid #222), icon kính lúp góc phải, loại bỏ nút xanh cồng kềnh, tích hợp live search AJAX</t>
         </is>
       </c>
       <c r="F49" s="79" t="inlineStr">
         <is>
-          <t>Khó</t>
-        </is>
-      </c>
-      <c r="G49" s="74" t="inlineStr">
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G49" s="83" t="inlineStr">
         <is>
           <t>Chờ thực hiện</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="28" customHeight="1">
+    <row r="50" ht="36" customHeight="1">
       <c r="A50" s="79" t="n">
         <v>3</v>
       </c>
       <c r="B50" s="80" t="inlineStr">
         <is>
-          <t>Main Navigation Bar (Thanh Menu Đỏ Đô &amp; Mega Menu)</t>
+          <t>Tái Cấu Trúc Cụm 4 Tiện Ích Bên Phải (Minimalist Header Icons)</t>
         </is>
       </c>
       <c r="C50" s="79" t="inlineStr">
         <is>
-          <t>WP Menu &amp; Customizer</t>
+          <t>Header Elements &amp; CSS</t>
         </is>
       </c>
       <c r="D50" s="80" t="inlineStr">
         <is>
-          <t>Flatsome Header Bottom</t>
+          <t>Flatsome Header &amp; style.css</t>
         </is>
       </c>
       <c r="E50" s="80" t="inlineStr">
         <is>
-          <t>Menu danh mục sản phẩm xe đạp trợ lực, mega menu dạng tabs/lưới ảnh, các trang tin tức &amp; chính sách</t>
+          <t>Bỏ 4 nút xanh cồng kềnh; chuyển sang phong cách Icon mảnh + Text 2 dòng tinh tế (Hotline Mua hàng, Cửa hàng gần bạn, Tài khoản tròn, Giỏ hàng 0 đ kèm giá)</t>
         </is>
       </c>
       <c r="F50" s="79" t="inlineStr">
         <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="G50" s="74" t="inlineStr">
+          <t>Khó</t>
+        </is>
+      </c>
+      <c r="G50" s="83" t="inlineStr">
         <is>
           <t>Chờ thực hiện</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="28" customHeight="1">
+    <row r="51" ht="36" customHeight="1">
       <c r="A51" s="79" t="n">
         <v>4</v>
       </c>
       <c r="B51" s="80" t="inlineStr">
         <is>
-          <t>Tổng Hợp &amp; Ghép Nối Các Nguồn Giao Diện</t>
+          <t>Chuẩn Hóa Menu Bar &amp; Khối DANH MỤC (Tầng 3)</t>
         </is>
       </c>
       <c r="C51" s="79" t="inlineStr">
         <is>
-          <t>Custom Shortcode/CSS</t>
+          <t>WP Menu &amp; Customizer</t>
         </is>
       </c>
       <c r="D51" s="80" t="inlineStr">
         <is>
-          <t>flatsome-child/functions.php</t>
+          <t>Flatsome Header Bottom &amp; CSS</t>
         </is>
       </c>
       <c r="E51" s="80" t="inlineStr">
         <is>
-          <t>Tiếp nhận tư liệu từ nhiều nguồn khác nhau của người dùng, chuẩn hóa màu sắc, font chữ và phong cách hiển thị đồng nhất</t>
+          <t>Đổi icon Danh mục sang lưới 4 ô vuông ⊞ kèm mũi tên; menu chữ hoa uppercase (Trang chủ, Giới thiệu, Sản phẩm, Tin tức, Liên hệ), thêm line ngăn cách mờ</t>
         </is>
       </c>
       <c r="F51" s="79" t="inlineStr">
         <is>
-          <t>Khó</t>
-        </is>
-      </c>
-      <c r="G51" s="74" t="inlineStr">
-        <is>
-          <t>Chờ tư liệu</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="28" customHeight="1">
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G51" s="83" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="36" customHeight="1">
       <c r="A52" s="79" t="n">
         <v>5</v>
       </c>
       <c r="B52" s="80" t="inlineStr">
         <is>
-          <t>Responsive Mobile Header (Menu Off-Canvas &amp; Sticky)</t>
+          <t>Kiểm Thử Responsive Mobile Header &amp; Sticky Navigation</t>
         </is>
       </c>
       <c r="C52" s="79" t="inlineStr">
         <is>
-          <t>Flatsome Mobile Header</t>
+          <t>Mobile Header &amp; CSS</t>
         </is>
       </c>
       <c r="D52" s="80" t="inlineStr">
         <is>
-          <t>Header Builder &amp; CSS</t>
+          <t>flatsome-child/style.css (Media Queries)</t>
         </is>
       </c>
       <c r="E52" s="80" t="inlineStr">
         <is>
-          <t>Tối ưu thanh header dính (sticky header), menu trượt off-canvas mượt mà trên điện thoại, thanh search mobile tiện lợi</t>
+          <t>Tối ưu thanh header dính (sticky header), menu trượt off-canvas mượt mà trên điện thoại, thanh search mobile gọn gàng, tránh tràn viền</t>
         </is>
       </c>
       <c r="F52" s="79" t="inlineStr">
@@ -4882,7 +4882,7 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G52" s="74" t="inlineStr">
+      <c r="G52" s="83" t="inlineStr">
         <is>
           <t>Chờ thực hiện</t>
         </is>

</xml_diff>

<commit_message>
feat: Cap nhat giao dien single product, lien ket local XAMPP va dong bo toan bo source code
</commit_message>
<xml_diff>
--- a/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
+++ b/wp-experience/2. Bảng theo dõi & nhập liệu thời gian công việc.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="32">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -203,8 +203,33 @@
       <color rgb="004B5563"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="10"/>
+    </font>
+    <font/>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="000F766E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -295,8 +320,14 @@
         <bgColor rgb="FFF3F4F6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFEFF6FF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -462,11 +493,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -689,6 +721,69 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="31" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="25" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1072,37 +1167,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>BẢNG THEO DÕI VÀ NHẬP LIỆU THỜI GIAN CÔNG VIỆC</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Dự án: GOBIKE (Xe Đạp Trợ Lực Điện) | Nền tảng: WordPress 6.x + Flatsome Theme (WooCommerce)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>STT</t>
@@ -1148,18 +1241,8 @@
           <t>Trạng Thái</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Độ Ưu Tiên</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Ghi Chú / Giải Pháp Kỹ Thuật</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
+    </row>
+    <row r="5">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -1202,18 +1285,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>WooCommerce Attributes (pa_pin, pa_dong-co, pa_quang-duong) + Danh mục xe</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
+    </row>
+    <row r="6">
       <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
@@ -1256,18 +1329,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="inlineStr">
-        <is>
-          <t>Flatsome Header Builder tùy biến màu sắc và bố cục</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+    </row>
+    <row r="7">
       <c r="A7" s="20" t="n">
         <v>3</v>
       </c>
@@ -1310,18 +1373,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>Menu màu đỏ #d0021b, liên kết danh mục xe trợ lực điện</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
+    </row>
+    <row r="8">
       <c r="A8" s="24" t="n">
         <v>4</v>
       </c>
@@ -1364,18 +1417,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J8" s="24" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K8" s="8" t="inlineStr">
-        <is>
-          <t>UX Builder chia cột 8/12 (Slider) và 4/12 (Tin tức &amp; Banner)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
+    </row>
+    <row r="9">
       <c r="A9" s="26" t="n">
         <v>5</v>
       </c>
@@ -1418,18 +1461,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J9" s="27" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>Lưới 5 sản phẩm Flash sale kèm thanh đo tiến độ bán hàng</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
+    </row>
+    <row r="10">
       <c r="A10" s="26" t="n">
         <v>6</v>
       </c>
@@ -1472,18 +1505,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J10" s="27" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>Shortcode [gobike_category_block] trong functions.php + CSS style.css</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
+    </row>
+    <row r="11">
       <c r="A11" s="10" t="n">
         <v>7</v>
       </c>
@@ -1526,18 +1549,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="K11" s="12" t="inlineStr">
-        <is>
-          <t>UX Builder Blog Posts element (4 posts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
+    </row>
+    <row r="12">
       <c r="A12" s="10" t="n">
         <v>8</v>
       </c>
@@ -1580,18 +1593,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="K12" s="12" t="inlineStr">
-        <is>
-          <t>17 Năm - Bảo hành 18T - Bảo dưỡng trọn đời - Giao 12h</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
+    </row>
+    <row r="13">
       <c r="A13" s="10" t="n">
         <v>9</v>
       </c>
@@ -1634,18 +1637,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J13" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K13" s="12" t="inlineStr">
-        <is>
-          <t>Flatsome Footer Builder + Widgets + Form đăng ký nhận tin</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
+    </row>
+    <row r="14">
       <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
@@ -1688,18 +1681,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K14" s="12" t="inlineStr">
-        <is>
-          <t>Media queries co giãn lưới sản phẩm và carousel mobile</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
+    </row>
+    <row r="15">
       <c r="A15" s="10" t="n">
         <v>11</v>
       </c>
@@ -1742,18 +1725,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J15" s="11" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="K15" s="12" t="inlineStr">
-        <is>
-          <t>Đã hiển thị chuẩn phân cấp Trang chủ / SẢN PHẨM tại đỉnh trang</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
+    </row>
+    <row r="16">
       <c r="A16" s="10" t="n">
         <v>12</v>
       </c>
@@ -1788,18 +1761,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J16" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K16" s="12" t="inlineStr">
-        <is>
-          <t>Đã hoàn thành: 2 Banner zoom từ tâm 0-&gt;1, cấu hình SCF Theme Settings</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
+    </row>
+    <row r="17">
       <c r="A17" s="10" t="n">
         <v>13</v>
       </c>
@@ -1842,18 +1805,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J17" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K17" s="12" t="inlineStr">
-        <is>
-          <t>Tích hợp sidebar filter-sidebar dạng dropdowns: Thương hiệu, Giá, Dòng xe, Bánh xe</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
+    </row>
+    <row r="18">
       <c r="A18" s="10" t="n">
         <v>14</v>
       </c>
@@ -1896,18 +1849,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J18" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K18" s="12" t="inlineStr">
-        <is>
-          <t>Tùy biến woocommerce_catalog_ordering thành cụm radio buttons trong khung viền xám</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
+    </row>
+    <row r="19">
       <c r="A19" s="10" t="n">
         <v>15</v>
       </c>
@@ -1942,18 +1885,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K19" s="12" t="inlineStr">
-        <is>
-          <t>Đã hoàn thành: Thuộc tính xe đạp, nhãn giảm giá ⚡ Giảm X%, lưới 5 cột hoàn chỉnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
+    </row>
+    <row r="20">
       <c r="A20" s="10" t="n">
         <v>16</v>
       </c>
@@ -1988,18 +1921,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="K20" s="12" t="inlineStr">
-        <is>
-          <t>Đã hoàn thành: Phân trang WooCommerce ô vuông đỏ bo góc chuẩn Flatsome</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
+    </row>
+    <row r="21">
       <c r="A21" s="10" t="n">
         <v>17</v>
       </c>
@@ -2034,18 +1957,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J21" s="11" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="K21" s="12" t="inlineStr">
-        <is>
-          <t>Đã hoàn thành: Tiêu đề viền nét đứt dashed #ccc, nội dung SCF Theme Settings</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
+    </row>
+    <row r="22">
       <c r="A22" s="10" t="n">
         <v>18</v>
       </c>
@@ -2080,18 +1993,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J22" s="11" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="K22" s="12" t="inlineStr">
-        <is>
-          <t>Đã hoàn thành: 4 cam kết dịch vụ chân trang chuẩn mockup</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
+    </row>
+    <row r="23">
       <c r="A23" s="10" t="n">
         <v>19</v>
       </c>
@@ -2126,18 +2029,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J23" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K23" s="12" t="inlineStr">
-        <is>
-          <t>Đã hoàn thành: Responsive mượt mà trên Mobile &amp; Tablet, tải trang nhanh</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="36" customHeight="1">
+    </row>
+    <row r="24">
       <c r="A24" s="10" t="n">
         <v>20</v>
       </c>
@@ -2180,18 +2073,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J24" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K24" s="51" t="inlineStr">
-        <is>
-          <t>Đóng gói toàn bộ logic PHP/CSS/JS bộ lọc vào 1 file gobike-product-filter.php; lọc 5 khoảng giá VNĐ; đồng bộ thanh sắp xếp radio; nạp ưu tiên đầu functions.php; push full repo GitHub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
+    </row>
+    <row r="25">
       <c r="A25" s="10" t="n">
         <v>21</v>
       </c>
@@ -2234,18 +2117,8 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J25" s="11" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K25" s="51" t="inlineStr">
-        <is>
-          <t>Khắc phục triệt để lỗi syntax chặn nạp SCF/Theme Settings; cấu hình 2 banner zoom từ tâm 0-&gt;1 và khối SEO chân trang kèm đường viền nét đứt chuẩn ảnh mockup; hoàn tất 100% trang Sản Phẩm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="42" customHeight="1">
+    </row>
+    <row r="26">
       <c r="A26" s="69" t="n">
         <v>22</v>
       </c>
@@ -2269,29 +2142,27 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="F26" s="70" t="n"/>
-      <c r="G26" s="70" t="n"/>
+      <c r="F26" s="70" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="G26" s="70" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
       <c r="H26" s="72">
         <f>IF(AND(F26&lt;&gt;"",G26&lt;&gt;""),(G26-F26)*24,"")</f>
         <v/>
       </c>
-      <c r="I26" s="74" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
-        </is>
-      </c>
-      <c r="J26" s="70" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K26" s="71" t="inlineStr">
-        <is>
-          <t>Triển khai 5 Subtask nâng cấp từ hiện trạng ảnh 2 đạt 100% chuẩn mẫu ảnh 1: Badges đỏ, box 4 showroom, tiện ích, hotline phân màu, logo BCT, form email.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="42" customHeight="1">
+      <c r="I26" s="54" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27" s="69" t="n">
         <v>23</v>
       </c>
@@ -2302,12 +2173,12 @@
       </c>
       <c r="C27" s="70" t="inlineStr">
         <is>
-          <t>Task HD-01</t>
+          <t>Task HD-01 (Header)</t>
         </is>
       </c>
       <c r="D27" s="71" t="inlineStr">
         <is>
-          <t>Tái cấu trúc Header theo chuẩn Flatsome mẫu (Ảnh 1): Khắc phục Top Bar lỗi shortcode, thay thế 4 nút xanh cồng kềnh bằng cụm Icon + Text 2 dòng tinh tế, thanh search viên thuốc viền mảnh và khối Menu Danh Mục lưới 4 ô vuông</t>
+          <t>Tái cấu trúc Header theo chuẩn Flatsome mẫu: Top Bar thông tin, thay 4 nút xanh bằng cụm Icon + Text 2 dòng, Menu Danh mục (Vertical Menu) &amp; hoàn thiện toàn bộ Header</t>
         </is>
       </c>
       <c r="E27" s="70" t="inlineStr">
@@ -2315,645 +2186,607 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="F27" s="70" t="n"/>
-      <c r="G27" s="70" t="n"/>
+      <c r="F27" s="70" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="G27" s="70" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
       <c r="H27" s="72">
         <f>IF(AND(F27&lt;&gt;"",G27&lt;&gt;""),(G27-F27)*24,"")</f>
         <v/>
       </c>
-      <c r="I27" s="74" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
-        </is>
-      </c>
-      <c r="J27" s="70" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="K27" s="71" t="inlineStr">
-        <is>
-          <t>Kế hoạch gồm 5 Subtask: Tối ưu Top Bar, Pill search bar, cụm 4 tiện ích Icon + Text 2 dòng, Menu Danh mục 4 ô vuông &amp; Responsive mobile. Dự toán: 2.5 - 3.5 giờ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="11" t="n"/>
-      <c r="F28" s="11" t="n"/>
-      <c r="G28" s="11" t="n"/>
-      <c r="H28" s="13">
+      <c r="I27" s="54" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="67" t="inlineStr">
+        <is>
+          <t>23.1</t>
+        </is>
+      </c>
+      <c r="B28" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C28" s="67" t="inlineStr">
+        <is>
+          <t>Task 2.1</t>
+        </is>
+      </c>
+      <c r="D28" s="59" t="inlineStr">
+        <is>
+          <t>Tùy biến Search Form Header: Xử lý gỡ bỏ CSS fix cứng kích thước, tinh chỉnh chiều rộng và giao diện khung tìm kiếm Flatsome Customizer</t>
+        </is>
+      </c>
+      <c r="E28" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F28" s="58" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="G28" s="58" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="H28" s="87">
         <f>IF(AND(F28&lt;&gt;"",G28&lt;&gt;""),(G28-F28)*24,"")</f>
         <v/>
       </c>
-      <c r="I28" s="11" t="n"/>
-      <c r="J28" s="11" t="n"/>
-      <c r="K28" s="12" t="n"/>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
-      <c r="H29" s="13">
+      <c r="I28" s="94" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="67" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C29" s="67" t="inlineStr">
+        <is>
+          <t>Task RP-01</t>
+        </is>
+      </c>
+      <c r="D29" s="59" t="inlineStr">
+        <is>
+          <t>Tối ưu hóa Responsive toàn diện Trang Chủ trên Mobile &amp; Tablet (Header mobile 2 tầng, Hero Slider, Flash Sale swipe tabs, 4 khối danh mục 2 cột, Tin tức &amp; Footer)</t>
+        </is>
+      </c>
+      <c r="E29" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F29" s="58" t="n"/>
+      <c r="G29" s="58" t="n"/>
+      <c r="H29" s="87">
         <f>IF(AND(F29&lt;&gt;"",G29&lt;&gt;""),(G29-F29)*24,"")</f>
         <v/>
       </c>
-      <c r="I29" s="11" t="n"/>
-      <c r="J29" s="11" t="n"/>
-      <c r="K29" s="12" t="n"/>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="I29" s="98" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="67" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C30" s="67" t="inlineStr">
+        <is>
+          <t>Task MB-01</t>
+        </is>
+      </c>
+      <c r="D30" s="59" t="inlineStr">
+        <is>
+          <t>Xây dựng Thanh Menu Dính Đáy Mobile (Mobile Bottom Navigation Bar) kèm Nút Hotline Tròn Nổi Bật (Raised Center FAB): 5 nút tiện ích (Trang chủ, Sản phẩm, Gọi điện, Messenger, Zalo)</t>
+        </is>
+      </c>
+      <c r="E30" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F30" s="58" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G30" s="58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="H30" s="58">
+        <f>IF(AND(F30&lt;&gt;"",G30&lt;&gt;""),(G30-F30)*24,"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="106" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="67" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C31" s="67" t="inlineStr">
+        <is>
+          <t>Task RP-01.2</t>
+        </is>
+      </c>
+      <c r="D31" s="59" t="inlineStr">
+        <is>
+          <t>Tối ưu Responsive Banner Slider Trang Chủ (Mobile &amp; Tablet): Ẩn 5 ô text thumbs, hiển thị thuần danh sách ảnh kèm Pagination dots viên thuốc đỏ/tròn xám chuẩn Sencom (page-blank.php &amp; style.css)</t>
+        </is>
+      </c>
+      <c r="E31" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F31" s="58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="G31" s="58" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="H31" s="58">
+        <f>IF(AND(F31&lt;&gt;"",G31&lt;&gt;""),(G31-F31)*24,"")</f>
+        <v/>
+      </c>
+      <c r="I31" s="106" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B32" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C32" s="67" t="inlineStr">
+        <is>
+          <t>Task RP-01.3</t>
+        </is>
+      </c>
+      <c r="D32" s="59" t="inlineStr">
+        <is>
+          <t>Tối ưu Banner Slider &amp; Khối Tin Tức Trang Chủ trên Desktop (Laptop &amp; PC): Cố định chiều cao ảnh slide 320px (object-fit: cover), 5 ô text 60px triệt tiêu khoảng trắng rỗng, cân bằng 2 khối Slider &amp; Tin tức 380px cả mép trên và đáy dưới (page-blank.php &amp; style.css)</t>
+        </is>
+      </c>
+      <c r="E32" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F32" s="58" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="G32" s="58" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="H32" s="58">
+        <f>IF(AND(F32&lt;&gt;"",G32&lt;&gt;""),(G32-F32)*24,"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="106" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>TỔNG CỘNG THỜI GIAN ĐÃ THỰC HIỆN (GIỜ):</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="19" t="n"/>
-      <c r="H30" s="16">
-        <f>SUM(H5:H29)</f>
+      <c r="B33" s="18" t="n"/>
+      <c r="C33" s="18" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="19" t="n"/>
+      <c r="H33" s="103">
+        <f>SUM(H5:H32)</f>
         <v/>
       </c>
-      <c r="I30" s="15" t="n"/>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="n"/>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="55" t="inlineStr">
+      <c r="I33" s="15" t="n"/>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="88" t="inlineStr">
         <is>
           <t>IV. BẢNG TỔNG KẾT THỜI GIAN THEO NGÀY (DAILY TIME TRACKING SUMMARY)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="56" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="56" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B33" s="56" t="inlineStr">
+      <c r="B36" s="56" t="inlineStr">
         <is>
           <t>Ngày Làm Việc</t>
         </is>
       </c>
-      <c r="C33" s="56" t="inlineStr">
+      <c r="C36" s="56" t="inlineStr">
         <is>
           <t>Số Lượng Task</t>
         </is>
       </c>
-      <c r="D33" s="57" t="inlineStr">
+      <c r="D36" s="57" t="inlineStr">
         <is>
           <t>Nội Dung Công Việc Trọng Tâm Trong Ngày</t>
         </is>
       </c>
-      <c r="E33" s="56" t="inlineStr">
+      <c r="E36" s="56" t="inlineStr">
         <is>
           <t>Người Phụ Trách</t>
         </is>
       </c>
-      <c r="F33" s="56" t="inlineStr">
+      <c r="F36" s="56" t="inlineStr">
         <is>
           <t>Khung Giờ Bắt Đầu</t>
         </is>
       </c>
-      <c r="G33" s="56" t="inlineStr">
+      <c r="G36" s="56" t="inlineStr">
         <is>
           <t>Khung Giờ Kết Thúc</t>
         </is>
       </c>
-      <c r="H33" s="56" t="inlineStr">
+      <c r="H36" s="56" t="inlineStr">
         <is>
           <t>Tổng Giờ (h)</t>
         </is>
       </c>
-      <c r="I33" s="56" t="inlineStr">
+      <c r="I36" s="56" t="inlineStr">
         <is>
           <t>Trạng Thái</t>
         </is>
       </c>
-      <c r="J33" s="56" t="inlineStr">
-        <is>
-          <t>Mức Độ Hoàn Thành</t>
-        </is>
-      </c>
-      <c r="K33" s="57" t="inlineStr">
-        <is>
-          <t>Đánh Giá Tiến Độ &amp; Kết Quả Bàn Giao</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="58" t="n">
+    </row>
+    <row r="37">
+      <c r="A37" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="B34" s="58" t="inlineStr">
+      <c r="B37" s="67" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="C34" s="58" t="inlineStr">
+      <c r="C37" s="58" t="inlineStr">
         <is>
           <t>13 Task</t>
         </is>
       </c>
-      <c r="D34" s="59" t="inlineStr">
+      <c r="D37" s="59" t="inlineStr">
         <is>
           <t>Khởi tạo Taxonomy/Attributes + Hoàn thành 10 Task Trang Chủ + Khởi động Trang Sản Phẩm (Breadcrumb, Bộ lọc, Sắp xếp)</t>
         </is>
       </c>
-      <c r="E34" s="58" t="inlineStr">
+      <c r="E37" s="58" t="inlineStr">
         <is>
           <t>Developer</t>
         </is>
       </c>
-      <c r="F34" s="58" t="inlineStr">
+      <c r="F37" s="58" t="inlineStr">
         <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="G34" s="58" t="inlineStr">
+      <c r="G37" s="58" t="inlineStr">
         <is>
           <t>21:45</t>
         </is>
       </c>
-      <c r="H34" s="58">
-        <f>SUMIF(B$5:B$29, "2026-09-07", H$5:H$29)</f>
+      <c r="H37" s="67" t="n">
+        <v>13</v>
+      </c>
+      <c r="I37" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="58" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="67" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C38" s="58" t="inlineStr">
+        <is>
+          <t>4 Task lớn</t>
+        </is>
+      </c>
+      <c r="D38" s="59" t="inlineStr">
+        <is>
+          <t>Hoàn tất 100% Trang Sản Phẩm (Task SP-01, SP-02) + Hoàn tất 100% Tái cấu trúc Header Flatsome (Task HD-01) + Hoàn tất 100% Footer 4 cột chuẩn mockup thương hiệu GoBike (Task FT-01)</t>
+        </is>
+      </c>
+      <c r="E38" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F38" s="58" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G38" s="58" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="H38" s="67" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="I38" s="60" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="B39" s="58" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C39" s="58" t="inlineStr">
+        <is>
+          <t>3 Task lớn</t>
+        </is>
+      </c>
+      <c r="D39" s="59" t="inlineStr">
+        <is>
+          <t>Menu Dính Đáy Mobile (Task MB-01) + Responsive Banner Slider Mobile Sencom (Task RP-01.2) + Tối ưu Banner Slider &amp; Khối Tin Tức Desktop bằng nhau 380px (Task RP-01.3)</t>
+        </is>
+      </c>
+      <c r="E39" s="58" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="F39" s="58" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G39" s="58" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="H39" s="67">
+        <f>SUM(H30:H32)</f>
         <v/>
       </c>
-      <c r="I34" s="60" t="inlineStr">
+      <c r="I39" s="102" t="inlineStr">
         <is>
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="J34" s="60" t="inlineStr">
-        <is>
-          <t>100% Đạt mục tiêu</t>
-        </is>
-      </c>
-      <c r="K34" s="59" t="inlineStr">
-        <is>
-          <t>Hoàn tất toàn bộ 10 khối Trang Chủ, cấu hình dữ liệu nền tảng và dựng khung sườn phân cấp Trang Sản Phẩm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="58" t="n">
+    </row>
+    <row r="40">
+      <c r="A40" s="61" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG THỜI GIAN LÀM VIỆC CẢ 3 NGÀY (GIỜ):</t>
+        </is>
+      </c>
+      <c r="B40" s="75" t="n"/>
+      <c r="C40" s="75" t="n"/>
+      <c r="D40" s="75" t="n"/>
+      <c r="E40" s="75" t="n"/>
+      <c r="F40" s="75" t="n"/>
+      <c r="G40" s="76" t="n"/>
+      <c r="H40" s="63">
+        <f>SUM(H37:H39)</f>
+        <v/>
+      </c>
+      <c r="I40" s="64" t="inlineStr">
+        <is>
+          <t>28.83 h</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="89" t="n"/>
+      <c r="B41" s="89" t="n"/>
+      <c r="C41" s="89" t="n"/>
+      <c r="D41" s="89" t="n"/>
+      <c r="E41" s="89" t="n"/>
+      <c r="F41" s="89" t="n"/>
+      <c r="G41" s="89" t="n"/>
+      <c r="H41" s="89" t="n"/>
+      <c r="I41" s="89" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="92" t="inlineStr">
+        <is>
+          <t>V. BẢNG TỔNG KẾT THỜI GIAN HOÀN THIỆN THEO TỪNG TASK NHỎ &amp; GIAI ĐOẠN (SUBTASK BREAKDOWN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="56" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B43" s="56" t="inlineStr">
+        <is>
+          <t>Mã Task</t>
+        </is>
+      </c>
+      <c r="C43" s="56" t="inlineStr">
+        <is>
+          <t>Giai Đoạn / Nhóm</t>
+        </is>
+      </c>
+      <c r="D43" s="57" t="inlineStr">
+        <is>
+          <t>Tên Task Nhỏ / Khối Giao Diện Cụ Thể</t>
+        </is>
+      </c>
+      <c r="E43" s="56" t="inlineStr">
+        <is>
+          <t>Công Cụ / File</t>
+        </is>
+      </c>
+      <c r="F43" s="56" t="inlineStr">
+        <is>
+          <t>Bắt Đầu</t>
+        </is>
+      </c>
+      <c r="G43" s="56" t="inlineStr">
+        <is>
+          <t>Kết Thúc</t>
+        </is>
+      </c>
+      <c r="H43" s="56" t="inlineStr">
+        <is>
+          <t>Số Giờ</t>
+        </is>
+      </c>
+      <c r="I43" s="56" t="inlineStr">
+        <is>
+          <t>Thời Lượng (Phút)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="67" t="inlineStr">
+        <is>
+          <t>Task 1</t>
+        </is>
+      </c>
+      <c r="C44" s="58" t="inlineStr">
+        <is>
+          <t>I. Nền Tảng</t>
+        </is>
+      </c>
+      <c r="D44" s="59" t="inlineStr">
+        <is>
+          <t>Khởi tạo Taxonomy danh mục xe &amp; Thuộc tính (Pin, Động cơ, Quãng đường, Tốc độ)</t>
+        </is>
+      </c>
+      <c r="E44" s="58" t="inlineStr">
+        <is>
+          <t>WP Admin &amp; Woo</t>
+        </is>
+      </c>
+      <c r="F44" s="58" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G44" s="58" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="H44" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="58" t="n">
         <v>2</v>
       </c>
-      <c r="B35" s="58" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="C35" s="58" t="inlineStr">
-        <is>
-          <t>2 Task lớn</t>
-        </is>
-      </c>
-      <c r="D35" s="59" t="inlineStr">
-        <is>
-          <t>Hoàn thiện Trang Sản Phẩm: Đóng gói gobike-product-filter.php (5 khoảng giá, sắp xếp radio, fix no-products), Cặp Banner zoom từ tâm, Khối SEO chân trang nét đứt, SCF Theme Settings &amp; Push GitHub</t>
-        </is>
-      </c>
-      <c r="E35" s="58" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="F35" s="58" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="G35" s="58" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="H35" s="58">
-        <f>SUMIF(B$5:B$29, "2026-09-08", H$5:H$29)</f>
-        <v/>
-      </c>
-      <c r="I35" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="J35" s="60" t="inlineStr">
-        <is>
-          <t>100% Đạt mục tiêu</t>
-        </is>
-      </c>
-      <c r="K35" s="59" t="inlineStr">
-        <is>
-          <t>Nghiệm thu trọn vẹn 100% Trang Sản Phẩm theo mockup; loại bỏ triệt để lỗi syntax chặn load code, đồng bộ mã nguồn lên Git.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="61" t="inlineStr">
-        <is>
-          <t>TỔNG CỘNG THỜI GIAN LÀM VIỆC CẢ 2 NGÀY (GIỜ):</t>
-        </is>
-      </c>
-      <c r="B36" s="75" t="n"/>
-      <c r="C36" s="75" t="n"/>
-      <c r="D36" s="75" t="n"/>
-      <c r="E36" s="75" t="n"/>
-      <c r="F36" s="75" t="n"/>
-      <c r="G36" s="76" t="n"/>
-      <c r="H36" s="63">
-        <f>SUM(H34:H35)</f>
-        <v/>
-      </c>
-      <c r="I36" s="64" t="inlineStr">
-        <is>
-          <t>100% XONG</t>
-        </is>
-      </c>
-      <c r="J36" s="64" t="inlineStr">
-        <is>
-          <t>ĐÚNG TIẾN ĐỘ</t>
-        </is>
-      </c>
-      <c r="K36" s="65" t="n"/>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="66" t="inlineStr">
-        <is>
-          <t>V. BẢNG TỔNG KẾT THỜI GIAN HOÀN THIỆN THEO TỪNG TASK NHỎ &amp; GIAI ĐOẠN (SUBTASK BREAKDOWN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="56" t="inlineStr">
-        <is>
-          <t>STT</t>
-        </is>
-      </c>
-      <c r="B39" s="56" t="inlineStr">
-        <is>
-          <t>Mã Task</t>
-        </is>
-      </c>
-      <c r="C39" s="56" t="inlineStr">
-        <is>
-          <t>Giai Đoạn / Nhóm</t>
-        </is>
-      </c>
-      <c r="D39" s="57" t="inlineStr">
-        <is>
-          <t>Tên Task Nhỏ / Khối Giao Diện Cụ Thể</t>
-        </is>
-      </c>
-      <c r="E39" s="56" t="inlineStr">
-        <is>
-          <t>Công Cụ / File Xử Lý</t>
-        </is>
-      </c>
-      <c r="F39" s="56" t="inlineStr">
-        <is>
-          <t>Bắt Đầu</t>
-        </is>
-      </c>
-      <c r="G39" s="56" t="inlineStr">
-        <is>
-          <t>Kết Thúc</t>
-        </is>
-      </c>
-      <c r="H39" s="56" t="inlineStr">
-        <is>
-          <t>Tổng Giờ (h)</t>
-        </is>
-      </c>
-      <c r="I39" s="56" t="inlineStr">
-        <is>
-          <t>Thời Lượng (Phút)</t>
-        </is>
-      </c>
-      <c r="J39" s="56" t="inlineStr">
-        <is>
-          <t>Trạng Thái</t>
-        </is>
-      </c>
-      <c r="K39" s="57" t="inlineStr">
-        <is>
-          <t>Kết Quả / Giá Trị Đạt Được</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="58" t="n">
-        <v>1</v>
-      </c>
-      <c r="B40" s="67" t="inlineStr">
-        <is>
-          <t>Task 1</t>
-        </is>
-      </c>
-      <c r="C40" s="58" t="inlineStr">
-        <is>
-          <t>I. Nền Tảng</t>
-        </is>
-      </c>
-      <c r="D40" s="59" t="inlineStr">
-        <is>
-          <t>Khởi tạo Taxonomy danh mục xe &amp; Thuộc tính (Pin, Động cơ, Quãng đường, Tốc độ)</t>
-        </is>
-      </c>
-      <c r="E40" s="58" t="inlineStr">
-        <is>
-          <t>WP Admin &amp; Woo</t>
-        </is>
-      </c>
-      <c r="F40" s="58" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="G40" s="58" t="inlineStr">
+      <c r="B45" s="67" t="inlineStr">
+        <is>
+          <t>Task 2</t>
+        </is>
+      </c>
+      <c r="C45" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D45" s="59" t="inlineStr">
+        <is>
+          <t>Header đa tầng: Topbar đỏ cam kết + Main Header đen + Live Search + Cụm Icons</t>
+        </is>
+      </c>
+      <c r="E45" s="58" t="inlineStr">
+        <is>
+          <t>Header Builder</t>
+        </is>
+      </c>
+      <c r="F45" s="58" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="H40" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="I40" s="58" t="inlineStr">
-        <is>
-          <t>60 phút</t>
-        </is>
-      </c>
-      <c r="J40" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K40" s="59" t="inlineStr">
-        <is>
-          <t>Cơ sở dữ liệu danh mục xe và bộ 4 thuộc tính kỹ thuật hoàn chỉnh</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="58" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="67" t="inlineStr">
-        <is>
-          <t>Task 2</t>
-        </is>
-      </c>
-      <c r="C41" s="58" t="inlineStr">
-        <is>
-          <t>II. Trang Chủ</t>
-        </is>
-      </c>
-      <c r="D41" s="59" t="inlineStr">
-        <is>
-          <t>Header đa tầng: Topbar đỏ cam kết + Main Header đen + Live Search + Cụm Icons</t>
-        </is>
-      </c>
-      <c r="E41" s="58" t="inlineStr">
-        <is>
-          <t>Header Builder</t>
-        </is>
-      </c>
-      <c r="F41" s="58" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="G41" s="58" t="inlineStr">
+      <c r="G45" s="58" t="inlineStr">
         <is>
           <t>10:30</t>
-        </is>
-      </c>
-      <c r="H41" s="67" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I41" s="58" t="inlineStr">
-        <is>
-          <t>90 phút</t>
-        </is>
-      </c>
-      <c r="J41" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K41" s="59" t="inlineStr">
-        <is>
-          <t>Header 2 tầng chuẩn nhận diện thương hiệu, AJAX live search sản phẩm</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="58" t="n">
-        <v>3</v>
-      </c>
-      <c r="B42" s="67" t="inlineStr">
-        <is>
-          <t>Task 3</t>
-        </is>
-      </c>
-      <c r="C42" s="58" t="inlineStr">
-        <is>
-          <t>II. Trang Chủ</t>
-        </is>
-      </c>
-      <c r="D42" s="59" t="inlineStr">
-        <is>
-          <t>Navigation Menu đỏ chính (#d0021b) + Tích hợp Mega Menu danh mục xe</t>
-        </is>
-      </c>
-      <c r="E42" s="58" t="inlineStr">
-        <is>
-          <t>WP Menu + CSS</t>
-        </is>
-      </c>
-      <c r="F42" s="58" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="G42" s="58" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="H42" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="58" t="inlineStr">
-        <is>
-          <t>60 phút</t>
-        </is>
-      </c>
-      <c r="J42" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K42" s="59" t="inlineStr">
-        <is>
-          <t>Thanh menu đỏ nổi bật, bo góc viền dưới, dropdown menu mượt mà</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="58" t="n">
-        <v>4</v>
-      </c>
-      <c r="B43" s="67" t="inlineStr">
-        <is>
-          <t>Task 4</t>
-        </is>
-      </c>
-      <c r="C43" s="58" t="inlineStr">
-        <is>
-          <t>II. Trang Chủ</t>
-        </is>
-      </c>
-      <c r="D43" s="59" t="inlineStr">
-        <is>
-          <t>Hero Section: Slider banner chính + Tin tức nổi bật + Banner giao hỏa tốc 1H</t>
-        </is>
-      </c>
-      <c r="E43" s="58" t="inlineStr">
-        <is>
-          <t>UX Builder</t>
-        </is>
-      </c>
-      <c r="F43" s="58" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="G43" s="58" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
-      <c r="H43" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="I43" s="58" t="inlineStr">
-        <is>
-          <t>60 phút</t>
-        </is>
-      </c>
-      <c r="J43" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K43" s="59" t="inlineStr">
-        <is>
-          <t>Bố cục 2/3 slider tự động chạy + 1/3 widget bài viết và banner cam</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="58" t="n">
-        <v>5</v>
-      </c>
-      <c r="B44" s="67" t="inlineStr">
-        <is>
-          <t>Task 5</t>
-        </is>
-      </c>
-      <c r="C44" s="58" t="inlineStr">
-        <is>
-          <t>II. Trang Chủ</t>
-        </is>
-      </c>
-      <c r="D44" s="59" t="inlineStr">
-        <is>
-          <t>Section Giờ Vàng - Giá Cực Sốc (Tabs 17h, 19h, 20h, 21h + Lưới 5 sản phẩm sale)</t>
-        </is>
-      </c>
-      <c r="E44" s="58" t="inlineStr">
-        <is>
-          <t>UX + Shortcode</t>
-        </is>
-      </c>
-      <c r="F44" s="58" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="G44" s="58" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
-      <c r="H44" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="I44" s="58" t="inlineStr">
-        <is>
-          <t>120 phút</t>
-        </is>
-      </c>
-      <c r="J44" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K44" s="59" t="inlineStr">
-        <is>
-          <t>Tabs mốc thời gian chuyển đổi nhanh, thanh tiến độ bán hàng trực quan</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="28" customHeight="1">
-      <c r="A45" s="58" t="n">
-        <v>6</v>
-      </c>
-      <c r="B45" s="67" t="inlineStr">
-        <is>
-          <t>Task 6</t>
-        </is>
-      </c>
-      <c r="C45" s="58" t="inlineStr">
-        <is>
-          <t>II. Trang Chủ</t>
-        </is>
-      </c>
-      <c r="D45" s="59" t="inlineStr">
-        <is>
-          <t>4 Khối danh mục xe đạp (Shortcode [gobike_category_block] lưới 5 cột: 1 Big + 8 Small)</t>
-        </is>
-      </c>
-      <c r="E45" s="58" t="inlineStr">
-        <is>
-          <t>functions.php &amp; CSS</t>
-        </is>
-      </c>
-      <c r="F45" s="58" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
-      <c r="G45" s="58" t="inlineStr">
-        <is>
-          <t>17:00</t>
         </is>
       </c>
       <c r="H45" s="67" t="n">
@@ -2964,24 +2797,14 @@
           <t>90 phút</t>
         </is>
       </c>
-      <c r="J45" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K45" s="59" t="inlineStr">
-        <is>
-          <t>Lưới 5 cột tự co giãn, tự tính nhãn ⚡ Giảm X%, in thông số pin/quãng đường</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="28" customHeight="1">
+    </row>
+    <row r="46">
       <c r="A46" s="58" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B46" s="67" t="inlineStr">
         <is>
-          <t>Task 7</t>
+          <t>Task 3</t>
         </is>
       </c>
       <c r="C46" s="58" t="inlineStr">
@@ -2991,22 +2814,22 @@
       </c>
       <c r="D46" s="59" t="inlineStr">
         <is>
-          <t>Section Tin tức - Bài viết Blog (Lưới 4 cột thumbnail, ngày đăng, tóm tắt)</t>
+          <t>Navigation Menu đỏ chính (#d0021b) + Tích hợp Mega Menu danh mục xe</t>
         </is>
       </c>
       <c r="E46" s="58" t="inlineStr">
         <is>
-          <t>UX Blog Posts</t>
+          <t>WP Menu &amp; CSS</t>
         </is>
       </c>
       <c r="F46" s="58" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="G46" s="58" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="H46" s="67" t="n">
@@ -3017,435 +2840,1190 @@
           <t>60 phút</t>
         </is>
       </c>
-      <c r="J46" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K46" s="59" t="inlineStr">
-        <is>
-          <t>Hiển thị 4 bài blog mới nhất, nút Xem tất cả liên kết trang tin</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="28" customHeight="1">
+    </row>
+    <row r="47">
       <c r="A47" s="58" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="67" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+      <c r="C47" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D47" s="59" t="inlineStr">
+        <is>
+          <t>Hero Section: Slider banner chính + Tin tức nổi bật + Banner giao hỏa tốc 1H</t>
+        </is>
+      </c>
+      <c r="E47" s="58" t="inlineStr">
+        <is>
+          <t>UX Builder</t>
+        </is>
+      </c>
+      <c r="F47" s="58" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G47" s="58" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="H47" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="58" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" s="67" t="inlineStr">
+        <is>
+          <t>Task 5</t>
+        </is>
+      </c>
+      <c r="C48" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D48" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section Giờ Vàng - Giá Cực Sốc (Tabs 17h, 19h, 20h, 21h + Lưới 5 sản phẩm sale) </t>
+        </is>
+      </c>
+      <c r="E48" s="58" t="inlineStr">
+        <is>
+          <t>UX &amp; Shortcode</t>
+        </is>
+      </c>
+      <c r="F48" s="58" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="G48" s="58" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="H48" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="I48" s="58" t="inlineStr">
+        <is>
+          <t>120 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="58" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" s="67" t="inlineStr">
+        <is>
+          <t>Task 6</t>
+        </is>
+      </c>
+      <c r="C49" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D49" s="59" t="inlineStr">
+        <is>
+          <t>4 Khối danh mục xe đạp (Shortcode [gobike_category_block] lưới 5 cột: 1 Big + 8 Small)</t>
+        </is>
+      </c>
+      <c r="E49" s="58" t="inlineStr">
+        <is>
+          <t>functions.php &amp; CSS</t>
+        </is>
+      </c>
+      <c r="F49" s="58" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="G49" s="58" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="H49" s="67" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I49" s="58" t="inlineStr">
+        <is>
+          <t>90 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="58" t="n">
+        <v>7</v>
+      </c>
+      <c r="B50" s="67" t="inlineStr">
+        <is>
+          <t>Task 7</t>
+        </is>
+      </c>
+      <c r="C50" s="58" t="inlineStr">
+        <is>
+          <t>II. Trang Chủ</t>
+        </is>
+      </c>
+      <c r="D50" s="59" t="inlineStr">
+        <is>
+          <t>Section Tin tức - Bài viết Blog (Lưới 4 cột thumbnail, ngày đăng, tóm tắt)</t>
+        </is>
+      </c>
+      <c r="E50" s="58" t="inlineStr">
+        <is>
+          <t>UX Blog Posts</t>
+        </is>
+      </c>
+      <c r="F50" s="58" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G50" s="58" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="H50" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" s="58" t="inlineStr">
+        <is>
+          <t>60 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="58" t="n">
         <v>8</v>
       </c>
-      <c r="B47" s="67" t="inlineStr">
+      <c r="B51" s="67" t="inlineStr">
         <is>
           <t>Task 8</t>
         </is>
       </c>
-      <c r="C47" s="58" t="inlineStr">
+      <c r="C51" s="58" t="inlineStr">
         <is>
           <t>II. Trang Chủ</t>
         </is>
       </c>
-      <c r="D47" s="59" t="inlineStr">
+      <c r="D51" s="59" t="inlineStr">
         <is>
           <t>Khối 4 Cam kết dịch vụ Trust Badges (17 Năm, 18T BH, Trọn đời, 12h Giao)</t>
         </is>
       </c>
-      <c r="E47" s="58" t="inlineStr">
+      <c r="E51" s="58" t="inlineStr">
         <is>
           <t>UX Icon Box Row</t>
         </is>
       </c>
-      <c r="F47" s="58" t="inlineStr">
+      <c r="F51" s="58" t="inlineStr">
         <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="G47" s="58" t="inlineStr">
+      <c r="G51" s="58" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="H47" s="67" t="n">
+      <c r="H51" s="67" t="n">
         <v>0.5</v>
       </c>
-      <c r="I47" s="58" t="inlineStr">
+      <c r="I51" s="58" t="inlineStr">
         <is>
           <t>30 phút</t>
         </is>
       </c>
-      <c r="J47" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K47" s="59" t="inlineStr">
-        <is>
-          <t>4 cam kết vàng bảo chứng thương hiệu, icon sắc nét chuẩn mockup</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="58" t="n">
+    </row>
+    <row r="52">
+      <c r="A52" s="58" t="n">
         <v>9</v>
       </c>
-      <c r="B48" s="67" t="inlineStr">
+      <c r="B52" s="67" t="inlineStr">
         <is>
           <t>Task 9</t>
         </is>
       </c>
-      <c r="C48" s="58" t="inlineStr">
+      <c r="C52" s="58" t="inlineStr">
         <is>
           <t>II. Trang Chủ</t>
         </is>
       </c>
-      <c r="D48" s="59" t="inlineStr">
+      <c r="D52" s="59" t="inlineStr">
         <is>
           <t>Footer 4 Cột hoàn chỉnh (Showroom, Chính sách, Bộ Công Thương, Thanh toán)</t>
         </is>
       </c>
-      <c r="E48" s="58" t="inlineStr">
+      <c r="E52" s="58" t="inlineStr">
         <is>
           <t>Flatsome Footer</t>
         </is>
       </c>
-      <c r="F48" s="58" t="inlineStr">
+      <c r="F52" s="58" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="G48" s="58" t="inlineStr">
+      <c r="G52" s="58" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="H48" s="67" t="n">
+      <c r="H52" s="67" t="n">
         <v>1.25</v>
       </c>
-      <c r="I48" s="58" t="inlineStr">
+      <c r="I52" s="58" t="inlineStr">
         <is>
           <t>75 phút</t>
         </is>
       </c>
-      <c r="J48" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K48" s="59" t="inlineStr">
-        <is>
-          <t>Chân trang đầy đủ thông tin pháp lý, bản quyền, địa chỉ showroom 3 miền</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="28" customHeight="1">
-      <c r="A49" s="58" t="n">
+    </row>
+    <row r="53">
+      <c r="A53" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="B49" s="67" t="inlineStr">
+      <c r="B53" s="67" t="inlineStr">
         <is>
           <t>Task 10</t>
         </is>
       </c>
-      <c r="C49" s="58" t="inlineStr">
+      <c r="C53" s="58" t="inlineStr">
         <is>
           <t>II. Trang Chủ</t>
         </is>
       </c>
-      <c r="D49" s="59" t="inlineStr">
+      <c r="D53" s="59" t="inlineStr">
         <is>
           <t>Kiểm thử Responsive Mobile/Tablet &amp; Tinh chỉnh hiển thị toàn bộ Trang Chủ</t>
         </is>
       </c>
-      <c r="E49" s="58" t="inlineStr">
+      <c r="E53" s="58" t="inlineStr">
         <is>
           <t>style.css &amp; QA</t>
         </is>
       </c>
-      <c r="F49" s="58" t="inlineStr">
+      <c r="F53" s="58" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="G49" s="58" t="inlineStr">
+      <c r="G53" s="58" t="inlineStr">
         <is>
           <t>21:45</t>
         </is>
       </c>
-      <c r="H49" s="67" t="n">
+      <c r="H53" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="I49" s="58" t="inlineStr">
+      <c r="I53" s="58" t="inlineStr">
         <is>
           <t>60 phút</t>
         </is>
       </c>
-      <c r="J49" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K49" s="59" t="inlineStr">
-        <is>
-          <t>Chuyển lưới 5 cột sang 2 cột trên điện thoại, menu mobile mượt mà</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="58" t="n">
+    </row>
+    <row r="54">
+      <c r="A54" s="58" t="n">
         <v>11</v>
       </c>
-      <c r="B50" s="67" t="inlineStr">
+      <c r="B54" s="67" t="inlineStr">
         <is>
           <t>Task 11</t>
         </is>
       </c>
-      <c r="C50" s="58" t="inlineStr">
+      <c r="C54" s="58" t="inlineStr">
         <is>
           <t>III. Trang SP</t>
         </is>
       </c>
-      <c r="D50" s="59" t="inlineStr">
+      <c r="D54" s="59" t="inlineStr">
         <is>
           <t>Breadcrumb điều hướng phân cấp (Trang chủ &gt; SẢN PHẨM / Tên danh mục xe)</t>
         </is>
       </c>
-      <c r="E50" s="58" t="inlineStr">
+      <c r="E54" s="58" t="inlineStr">
         <is>
           <t>category-none.php</t>
         </is>
       </c>
-      <c r="F50" s="58" t="inlineStr">
+      <c r="F54" s="58" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="G50" s="58" t="inlineStr">
+      <c r="G54" s="58" t="inlineStr">
         <is>
           <t>16:25</t>
         </is>
       </c>
-      <c r="H50" s="67" t="n">
+      <c r="H54" s="67" t="n">
         <v>0.42</v>
       </c>
-      <c r="I50" s="58" t="inlineStr">
+      <c r="I54" s="58" t="inlineStr">
         <is>
           <t>25 phút</t>
         </is>
       </c>
-      <c r="J50" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K50" s="59" t="inlineStr">
-        <is>
-          <t>Thanh điều hướng phân cấp chuẩn SEO, font 13px xám nhạt tại đỉnh trang</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="58" t="n">
+    </row>
+    <row r="55">
+      <c r="A55" s="58" t="n">
         <v>12</v>
       </c>
-      <c r="B51" s="67" t="inlineStr">
+      <c r="B55" s="67" t="inlineStr">
         <is>
           <t>Task 13+14+SP1</t>
         </is>
       </c>
-      <c r="C51" s="58" t="inlineStr">
+      <c r="C55" s="58" t="inlineStr">
         <is>
           <t>III. Trang SP</t>
         </is>
       </c>
-      <c r="D51" s="59" t="inlineStr">
+      <c r="D55" s="59" t="inlineStr">
         <is>
           <t>Module Bộ Lọc Ngang độc lập (gobike-product-filter.php), 5 Khoảng Giá, Sắp xếp radio</t>
         </is>
       </c>
-      <c r="E51" s="58" t="inlineStr">
+      <c r="E55" s="58" t="inlineStr">
         <is>
           <t>gobike-product-filter.php</t>
         </is>
       </c>
-      <c r="F51" s="58" t="inlineStr">
+      <c r="F55" s="58" t="inlineStr">
         <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="G51" s="58" t="inlineStr">
+      <c r="G55" s="58" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="H51" s="67" t="n">
+      <c r="H55" s="67" t="n">
         <v>2.33</v>
       </c>
-      <c r="I51" s="58" t="inlineStr">
+      <c r="I55" s="58" t="inlineStr">
         <is>
           <t>140 phút</t>
         </is>
       </c>
-      <c r="J51" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K51" s="59" t="inlineStr">
-        <is>
-          <t>Gói gọn 100% PHP/CSS/JS 1 file; 5 nấc giá VNĐ; nút Bỏ bộ lọc; no-products chuẩn</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="28" customHeight="1">
-      <c r="A52" s="58" t="n">
+    </row>
+    <row r="56">
+      <c r="A56" s="58" t="n">
         <v>13</v>
       </c>
-      <c r="B52" s="67" t="inlineStr">
+      <c r="B56" s="67" t="inlineStr">
         <is>
           <t>Task 12+17+SP2</t>
         </is>
       </c>
-      <c r="C52" s="58" t="inlineStr">
+      <c r="C56" s="58" t="inlineStr">
         <is>
           <t>III. Trang SP</t>
         </is>
       </c>
-      <c r="D52" s="59" t="inlineStr">
+      <c r="D56" s="59" t="inlineStr">
         <is>
           <t>Cặp Banner zoom từ tâm (0-&gt;1) + Khối SEO chân trang nét đứt + Tích hợp SCF Theme Settings</t>
         </is>
       </c>
-      <c r="E52" s="58" t="inlineStr">
+      <c r="E56" s="58" t="inlineStr">
         <is>
           <t>functions.php &amp; CSS</t>
         </is>
       </c>
-      <c r="F52" s="58" t="inlineStr">
+      <c r="F56" s="58" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="G52" s="58" t="inlineStr">
+      <c r="G56" s="58" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="H52" s="67" t="n">
+      <c r="H56" s="67" t="n">
         <v>1.75</v>
       </c>
-      <c r="I52" s="58" t="inlineStr">
+      <c r="I56" s="58" t="inlineStr">
         <is>
           <t>105 phút</t>
         </is>
       </c>
-      <c r="J52" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K52" s="59" t="inlineStr">
-        <is>
-          <t>2 Banner zoom animation trung tâm; tiêu đề SEO gạch nét đứt #ccc; fix bug functions.php</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="58" t="n">
+    </row>
+    <row r="57">
+      <c r="A57" s="58" t="n">
         <v>14</v>
       </c>
-      <c r="B53" s="67" t="inlineStr">
+      <c r="B57" s="67" t="inlineStr">
         <is>
           <t>Task 15-19</t>
         </is>
       </c>
-      <c r="C53" s="58" t="inlineStr">
+      <c r="C57" s="58" t="inlineStr">
         <is>
           <t>III. Trang SP</t>
         </is>
       </c>
-      <c r="D53" s="59" t="inlineStr">
+      <c r="D57" s="59" t="inlineStr">
         <is>
           <t>Đồng bộ Card sản phẩm xe đạp, Phân trang đỏ bo góc, 4 Badges &amp; Responsive Trang SP</t>
         </is>
       </c>
-      <c r="E53" s="58" t="inlineStr">
+      <c r="E57" s="58" t="inlineStr">
         <is>
           <t>category-none.php &amp; CSS</t>
         </is>
       </c>
-      <c r="F53" s="58" t="inlineStr">
+      <c r="F57" s="58" t="inlineStr">
         <is>
           <t>Tích hợp</t>
         </is>
       </c>
-      <c r="G53" s="58" t="inlineStr">
+      <c r="G57" s="58" t="inlineStr">
         <is>
           <t>Đồng bộ</t>
         </is>
       </c>
-      <c r="H53" s="67" t="n">
+      <c r="H57" s="67" t="n">
         <v>0</v>
       </c>
-      <c r="I53" s="58" t="inlineStr">
+      <c r="I57" s="58" t="inlineStr">
         <is>
           <t>Đã tích hợp</t>
         </is>
       </c>
-      <c r="J53" s="60" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="K53" s="59" t="inlineStr">
-        <is>
-          <t>Hoàn thành 100% giao diện Catalog Archive chuẩn mockup, pixel-perfect</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="61" t="inlineStr">
+    </row>
+    <row r="58">
+      <c r="A58" s="58" t="n">
+        <v>15</v>
+      </c>
+      <c r="B58" s="67" t="inlineStr">
+        <is>
+          <t>Task 2.1</t>
+        </is>
+      </c>
+      <c r="C58" s="58" t="inlineStr">
+        <is>
+          <t>IV. Header Flatsome</t>
+        </is>
+      </c>
+      <c r="D58" s="59" t="inlineStr">
+        <is>
+          <t>Tùy biến Search Form Header: Gỡ bỏ CSS fix cứng kích thước, tinh chỉnh chiều rộng &amp; tỷ lệ co giãn Customizer</t>
+        </is>
+      </c>
+      <c r="E58" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Search &amp; CSS</t>
+        </is>
+      </c>
+      <c r="F58" s="58" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="G58" s="58" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="H58" s="67" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="I58" s="58" t="inlineStr">
+        <is>
+          <t>35 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="58" t="n">
+        <v>16</v>
+      </c>
+      <c r="B59" s="67" t="inlineStr">
+        <is>
+          <t>Task HD-01</t>
+        </is>
+      </c>
+      <c r="C59" s="58" t="inlineStr">
+        <is>
+          <t>IV. Header Flatsome</t>
+        </is>
+      </c>
+      <c r="D59" s="59" t="inlineStr">
+        <is>
+          <t>Tái cấu trúc Header toàn diện: Top Bar, Cụm 4 icons tinh tế, Vertical Menu &amp; CSS</t>
+        </is>
+      </c>
+      <c r="E59" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Header Builder</t>
+        </is>
+      </c>
+      <c r="F59" s="58" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="G59" s="58" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="H59" s="67" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I59" s="58" t="inlineStr">
+        <is>
+          <t>105 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="58" t="n">
+        <v>17</v>
+      </c>
+      <c r="B60" s="67" t="inlineStr">
+        <is>
+          <t>Task FT-01</t>
+        </is>
+      </c>
+      <c r="C60" s="58" t="inlineStr">
+        <is>
+          <t>V. Footer GoBike</t>
+        </is>
+      </c>
+      <c r="D60" s="59" t="inlineStr">
+        <is>
+          <t>Xây dựng Footer 4 cột chuẩn mockup GoBike: Box 3 Showroom, Thanh toán, Tiện ích, 5 Hotline, MXH, Fanpage &amp; Form nhận tin</t>
+        </is>
+      </c>
+      <c r="E60" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Footer / UX Block</t>
+        </is>
+      </c>
+      <c r="F60" s="58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="G60" s="58" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="H60" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="I60" s="58" t="inlineStr">
+        <is>
+          <t>180 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="B61" s="67" t="inlineStr">
+        <is>
+          <t>Task MB-01</t>
+        </is>
+      </c>
+      <c r="C61" s="58" t="inlineStr">
+        <is>
+          <t>VI. Mobile Bottom Bar</t>
+        </is>
+      </c>
+      <c r="D61" s="59" t="inlineStr">
+        <is>
+          <t>Xây dựng Mobile Bottom Navigation Bar 5 nút tiện ích kèm Nút Hotline Tròn Nổi Bật ở giữa (Raised Center FAB)</t>
+        </is>
+      </c>
+      <c r="E61" s="104" t="inlineStr">
+        <is>
+          <t>flatsome-child/functions.php &amp; style.css</t>
+        </is>
+      </c>
+      <c r="F61" s="58" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G61" s="58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="H61" s="67" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="I61" s="102" t="inlineStr">
+        <is>
+          <t>275 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="67" t="n">
+        <v>19</v>
+      </c>
+      <c r="B62" s="67" t="inlineStr">
+        <is>
+          <t>Task RP-01.2</t>
+        </is>
+      </c>
+      <c r="C62" s="58" t="inlineStr">
+        <is>
+          <t>VII. Responsive Banner</t>
+        </is>
+      </c>
+      <c r="D62" s="59" t="inlineStr">
+        <is>
+          <t>Tối ưu Responsive Banner Slider Trang Chủ (Mobile &amp; Tablet): Ẩn 5 thumbs, hiển thị dots đỏ/xám Sencom</t>
+        </is>
+      </c>
+      <c r="E62" s="104" t="inlineStr">
+        <is>
+          <t>page-blank.php &amp; style.css</t>
+        </is>
+      </c>
+      <c r="F62" s="58" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="G62" s="58" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="H62" s="67" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I62" s="102" t="inlineStr">
+        <is>
+          <t>20 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="67" t="n">
+        <v>20</v>
+      </c>
+      <c r="B63" s="67" t="inlineStr">
+        <is>
+          <t>Task RP-01.3</t>
+        </is>
+      </c>
+      <c r="C63" s="58" t="inlineStr">
+        <is>
+          <t>VII. Banner Desktop</t>
+        </is>
+      </c>
+      <c r="D63" s="59" t="inlineStr">
+        <is>
+          <t>Tối ưu Banner Slider &amp; Cân Bằng Khối Tin Tức Desktop: Cố định 320px cover, xóa khoảng trắng, cân bằng 380px</t>
+        </is>
+      </c>
+      <c r="E63" s="104" t="inlineStr">
+        <is>
+          <t>style.css &amp; page-blank.php</t>
+        </is>
+      </c>
+      <c r="F63" s="58" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="G63" s="58" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="H63" s="67" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="I63" s="102" t="inlineStr">
+        <is>
+          <t>140 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="61" t="inlineStr">
         <is>
           <t>TỔNG THỜI GIAN HOÀN THIỆN TẤT CẢ CÁC TASK NHỎ (GIỜ):</t>
         </is>
       </c>
-      <c r="B54" s="75" t="n"/>
-      <c r="C54" s="75" t="n"/>
-      <c r="D54" s="75" t="n"/>
-      <c r="E54" s="75" t="n"/>
-      <c r="F54" s="75" t="n"/>
-      <c r="G54" s="76" t="n"/>
-      <c r="H54" s="63">
-        <f>SUM(H40:H53)</f>
+      <c r="B64" s="75" t="n"/>
+      <c r="C64" s="75" t="n"/>
+      <c r="D64" s="75" t="n"/>
+      <c r="E64" s="75" t="n"/>
+      <c r="F64" s="75" t="n"/>
+      <c r="G64" s="76" t="n"/>
+      <c r="H64" s="63">
+        <f>SUM(H44:H63)</f>
         <v/>
       </c>
-      <c r="I54" s="63" t="inlineStr">
-        <is>
-          <t>975 Phút (~16.25h)</t>
-        </is>
-      </c>
-      <c r="J54" s="64" t="inlineStr">
-        <is>
-          <t>100% HOÀN THÀNH</t>
-        </is>
-      </c>
-      <c r="K54" s="68" t="inlineStr">
-        <is>
-          <t>Đã nghiệm thu toàn diện Trang Chủ &amp; Trang Sản Phẩm</t>
-        </is>
-      </c>
+      <c r="I64" s="63" t="inlineStr">
+        <is>
+          <t>1730 Phút (~28.83h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="89" t="n"/>
+      <c r="B65" s="89" t="n"/>
+      <c r="C65" s="89" t="n"/>
+      <c r="D65" s="89" t="n"/>
+      <c r="E65" s="89" t="n"/>
+      <c r="F65" s="89" t="n"/>
+      <c r="G65" s="89" t="n"/>
+      <c r="H65" s="89" t="n"/>
+      <c r="I65" s="89" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="89" t="n"/>
+      <c r="B66" s="89" t="n"/>
+      <c r="C66" s="89" t="n"/>
+      <c r="D66" s="89" t="n"/>
+      <c r="E66" s="89" t="n"/>
+      <c r="F66" s="89" t="n"/>
+      <c r="G66" s="89" t="n"/>
+      <c r="H66" s="89" t="n"/>
+      <c r="I66" s="89" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="89" t="n"/>
+      <c r="B67" s="89" t="n"/>
+      <c r="C67" s="89" t="n"/>
+      <c r="D67" s="89" t="n"/>
+      <c r="E67" s="89" t="n"/>
+      <c r="F67" s="89" t="n"/>
+      <c r="G67" s="89" t="n"/>
+      <c r="H67" s="89" t="n"/>
+      <c r="I67" s="89" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="89" t="n"/>
+      <c r="B68" s="89" t="n"/>
+      <c r="C68" s="89" t="n"/>
+      <c r="D68" s="89" t="n"/>
+      <c r="E68" s="89" t="n"/>
+      <c r="F68" s="89" t="n"/>
+      <c r="G68" s="89" t="n"/>
+      <c r="H68" s="89" t="n"/>
+      <c r="I68" s="89" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="89" t="n"/>
+      <c r="B69" s="89" t="n"/>
+      <c r="C69" s="89" t="n"/>
+      <c r="D69" s="89" t="n"/>
+      <c r="E69" s="89" t="n"/>
+      <c r="F69" s="89" t="n"/>
+      <c r="G69" s="89" t="n"/>
+      <c r="H69" s="89" t="n"/>
+      <c r="I69" s="89" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="89" t="n"/>
+      <c r="B70" s="89" t="n"/>
+      <c r="C70" s="89" t="n"/>
+      <c r="D70" s="89" t="n"/>
+      <c r="E70" s="89" t="n"/>
+      <c r="F70" s="89" t="n"/>
+      <c r="G70" s="89" t="n"/>
+      <c r="H70" s="89" t="n"/>
+      <c r="I70" s="89" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="89" t="n"/>
+      <c r="B71" s="89" t="n"/>
+      <c r="C71" s="89" t="n"/>
+      <c r="D71" s="89" t="n"/>
+      <c r="E71" s="89" t="n"/>
+      <c r="F71" s="89" t="n"/>
+      <c r="G71" s="89" t="n"/>
+      <c r="H71" s="89" t="n"/>
+      <c r="I71" s="89" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="89" t="n"/>
+      <c r="B72" s="89" t="n"/>
+      <c r="C72" s="89" t="n"/>
+      <c r="D72" s="89" t="n"/>
+      <c r="E72" s="89" t="n"/>
+      <c r="F72" s="89" t="n"/>
+      <c r="G72" s="89" t="n"/>
+      <c r="H72" s="89" t="n"/>
+      <c r="I72" s="89" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="89" t="n"/>
+      <c r="B73" s="89" t="n"/>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="89" t="n"/>
+      <c r="F73" s="89" t="n"/>
+      <c r="G73" s="89" t="n"/>
+      <c r="H73" s="89" t="n"/>
+      <c r="I73" s="89" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="89" t="n"/>
+      <c r="B74" s="89" t="n"/>
+      <c r="C74" s="89" t="n"/>
+      <c r="D74" s="89" t="n"/>
+      <c r="E74" s="89" t="n"/>
+      <c r="F74" s="89" t="n"/>
+      <c r="G74" s="89" t="n"/>
+      <c r="H74" s="89" t="n"/>
+      <c r="I74" s="89" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="89" t="n"/>
+      <c r="B75" s="89" t="n"/>
+      <c r="C75" s="89" t="n"/>
+      <c r="D75" s="89" t="n"/>
+      <c r="E75" s="89" t="n"/>
+      <c r="F75" s="89" t="n"/>
+      <c r="G75" s="89" t="n"/>
+      <c r="H75" s="89" t="n"/>
+      <c r="I75" s="89" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="89" t="n"/>
+      <c r="B76" s="89" t="n"/>
+      <c r="C76" s="89" t="n"/>
+      <c r="D76" s="89" t="n"/>
+      <c r="E76" s="89" t="n"/>
+      <c r="F76" s="89" t="n"/>
+      <c r="G76" s="89" t="n"/>
+      <c r="H76" s="89" t="n"/>
+      <c r="I76" s="89" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="89" t="n"/>
+      <c r="B77" s="89" t="n"/>
+      <c r="C77" s="89" t="n"/>
+      <c r="D77" s="89" t="n"/>
+      <c r="E77" s="89" t="n"/>
+      <c r="F77" s="89" t="n"/>
+      <c r="G77" s="89" t="n"/>
+      <c r="H77" s="89" t="n"/>
+      <c r="I77" s="89" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="89" t="n"/>
+      <c r="B78" s="89" t="n"/>
+      <c r="C78" s="89" t="n"/>
+      <c r="D78" s="89" t="n"/>
+      <c r="E78" s="89" t="n"/>
+      <c r="F78" s="89" t="n"/>
+      <c r="G78" s="89" t="n"/>
+      <c r="H78" s="89" t="n"/>
+      <c r="I78" s="89" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="89" t="n"/>
+      <c r="B79" s="89" t="n"/>
+      <c r="C79" s="89" t="n"/>
+      <c r="D79" s="89" t="n"/>
+      <c r="E79" s="89" t="n"/>
+      <c r="F79" s="89" t="n"/>
+      <c r="G79" s="89" t="n"/>
+      <c r="H79" s="89" t="n"/>
+      <c r="I79" s="89" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="89" t="n"/>
+      <c r="B80" s="89" t="n"/>
+      <c r="C80" s="89" t="n"/>
+      <c r="D80" s="89" t="n"/>
+      <c r="E80" s="89" t="n"/>
+      <c r="F80" s="89" t="n"/>
+      <c r="G80" s="89" t="n"/>
+      <c r="H80" s="89" t="n"/>
+      <c r="I80" s="89" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="89" t="n"/>
+      <c r="B81" s="89" t="n"/>
+      <c r="C81" s="89" t="n"/>
+      <c r="D81" s="89" t="n"/>
+      <c r="E81" s="89" t="n"/>
+      <c r="F81" s="89" t="n"/>
+      <c r="G81" s="89" t="n"/>
+      <c r="H81" s="89" t="n"/>
+      <c r="I81" s="89" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="89" t="n"/>
+      <c r="B82" s="89" t="n"/>
+      <c r="C82" s="89" t="n"/>
+      <c r="D82" s="89" t="n"/>
+      <c r="E82" s="89" t="n"/>
+      <c r="F82" s="89" t="n"/>
+      <c r="G82" s="89" t="n"/>
+      <c r="H82" s="89" t="n"/>
+      <c r="I82" s="89" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="89" t="n"/>
+      <c r="B83" s="89" t="n"/>
+      <c r="C83" s="89" t="n"/>
+      <c r="D83" s="89" t="n"/>
+      <c r="E83" s="89" t="n"/>
+      <c r="F83" s="89" t="n"/>
+      <c r="G83" s="89" t="n"/>
+      <c r="H83" s="89" t="n"/>
+      <c r="I83" s="89" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="89" t="n"/>
+      <c r="B84" s="89" t="n"/>
+      <c r="C84" s="89" t="n"/>
+      <c r="D84" s="89" t="n"/>
+      <c r="E84" s="89" t="n"/>
+      <c r="F84" s="89" t="n"/>
+      <c r="G84" s="89" t="n"/>
+      <c r="H84" s="89" t="n"/>
+      <c r="I84" s="89" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="89" t="n"/>
+      <c r="B85" s="89" t="n"/>
+      <c r="C85" s="89" t="n"/>
+      <c r="D85" s="89" t="n"/>
+      <c r="E85" s="89" t="n"/>
+      <c r="F85" s="89" t="n"/>
+      <c r="G85" s="89" t="n"/>
+      <c r="H85" s="89" t="n"/>
+      <c r="I85" s="89" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="89" t="n"/>
+      <c r="B86" s="89" t="n"/>
+      <c r="C86" s="89" t="n"/>
+      <c r="D86" s="89" t="n"/>
+      <c r="E86" s="89" t="n"/>
+      <c r="F86" s="89" t="n"/>
+      <c r="G86" s="89" t="n"/>
+      <c r="H86" s="89" t="n"/>
+      <c r="I86" s="89" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="89" t="n"/>
+      <c r="B87" s="89" t="n"/>
+      <c r="C87" s="89" t="n"/>
+      <c r="D87" s="89" t="n"/>
+      <c r="E87" s="89" t="n"/>
+      <c r="F87" s="89" t="n"/>
+      <c r="G87" s="89" t="n"/>
+      <c r="H87" s="89" t="n"/>
+      <c r="I87" s="89" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="89" t="n"/>
+      <c r="B88" s="89" t="n"/>
+      <c r="C88" s="89" t="n"/>
+      <c r="D88" s="89" t="n"/>
+      <c r="E88" s="89" t="n"/>
+      <c r="F88" s="89" t="n"/>
+      <c r="G88" s="89" t="n"/>
+      <c r="H88" s="89" t="n"/>
+      <c r="I88" s="89" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="89" t="n"/>
+      <c r="B89" s="89" t="n"/>
+      <c r="C89" s="89" t="n"/>
+      <c r="D89" s="89" t="n"/>
+      <c r="E89" s="89" t="n"/>
+      <c r="F89" s="89" t="n"/>
+      <c r="G89" s="89" t="n"/>
+      <c r="H89" s="89" t="n"/>
+      <c r="I89" s="89" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="89" t="n"/>
+      <c r="B90" s="89" t="n"/>
+      <c r="C90" s="89" t="n"/>
+      <c r="D90" s="89" t="n"/>
+      <c r="E90" s="89" t="n"/>
+      <c r="F90" s="89" t="n"/>
+      <c r="G90" s="89" t="n"/>
+      <c r="H90" s="89" t="n"/>
+      <c r="I90" s="89" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="89" t="n"/>
+      <c r="B91" s="89" t="n"/>
+      <c r="C91" s="89" t="n"/>
+      <c r="D91" s="89" t="n"/>
+      <c r="E91" s="89" t="n"/>
+      <c r="F91" s="89" t="n"/>
+      <c r="G91" s="89" t="n"/>
+      <c r="H91" s="89" t="n"/>
+      <c r="I91" s="89" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="89" t="n"/>
+      <c r="B92" s="89" t="n"/>
+      <c r="C92" s="89" t="n"/>
+      <c r="D92" s="89" t="n"/>
+      <c r="E92" s="89" t="n"/>
+      <c r="F92" s="89" t="n"/>
+      <c r="G92" s="89" t="n"/>
+      <c r="H92" s="89" t="n"/>
+      <c r="I92" s="89" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="89" t="n"/>
+      <c r="B93" s="89" t="n"/>
+      <c r="C93" s="89" t="n"/>
+      <c r="D93" s="89" t="n"/>
+      <c r="E93" s="89" t="n"/>
+      <c r="F93" s="89" t="n"/>
+      <c r="G93" s="89" t="n"/>
+      <c r="H93" s="89" t="n"/>
+      <c r="I93" s="89" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="89" t="n"/>
+      <c r="B94" s="89" t="n"/>
+      <c r="C94" s="89" t="n"/>
+      <c r="D94" s="89" t="n"/>
+      <c r="E94" s="89" t="n"/>
+      <c r="F94" s="89" t="n"/>
+      <c r="G94" s="89" t="n"/>
+      <c r="H94" s="89" t="n"/>
+      <c r="I94" s="89" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="89" t="n"/>
+      <c r="B95" s="89" t="n"/>
+      <c r="C95" s="89" t="n"/>
+      <c r="D95" s="89" t="n"/>
+      <c r="E95" s="89" t="n"/>
+      <c r="F95" s="89" t="n"/>
+      <c r="G95" s="89" t="n"/>
+      <c r="H95" s="89" t="n"/>
+      <c r="I95" s="89" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="89" t="n"/>
+      <c r="B96" s="89" t="n"/>
+      <c r="C96" s="89" t="n"/>
+      <c r="D96" s="89" t="n"/>
+      <c r="E96" s="89" t="n"/>
+      <c r="F96" s="89" t="n"/>
+      <c r="G96" s="89" t="n"/>
+      <c r="H96" s="89" t="n"/>
+      <c r="I96" s="89" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="89" t="n"/>
+      <c r="B97" s="89" t="n"/>
+      <c r="C97" s="89" t="n"/>
+      <c r="D97" s="89" t="n"/>
+      <c r="E97" s="89" t="n"/>
+      <c r="F97" s="89" t="n"/>
+      <c r="G97" s="89" t="n"/>
+      <c r="H97" s="89" t="n"/>
+      <c r="I97" s="89" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="89" t="n"/>
+      <c r="B98" s="89" t="n"/>
+      <c r="C98" s="89" t="n"/>
+      <c r="D98" s="89" t="n"/>
+      <c r="E98" s="89" t="n"/>
+      <c r="F98" s="89" t="n"/>
+      <c r="G98" s="89" t="n"/>
+      <c r="H98" s="89" t="n"/>
+      <c r="I98" s="89" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="89" t="n"/>
+      <c r="B99" s="89" t="n"/>
+      <c r="C99" s="89" t="n"/>
+      <c r="D99" s="89" t="n"/>
+      <c r="E99" s="89" t="n"/>
+      <c r="F99" s="89" t="n"/>
+      <c r="G99" s="89" t="n"/>
+      <c r="H99" s="89" t="n"/>
+      <c r="I99" s="89" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="89" t="n"/>
+      <c r="B100" s="89" t="n"/>
+      <c r="C100" s="89" t="n"/>
+      <c r="D100" s="89" t="n"/>
+      <c r="E100" s="89" t="n"/>
+      <c r="F100" s="89" t="n"/>
+      <c r="G100" s="89" t="n"/>
+      <c r="H100" s="89" t="n"/>
+      <c r="I100" s="89" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="89" t="n"/>
+      <c r="B101" s="89" t="n"/>
+      <c r="C101" s="89" t="n"/>
+      <c r="D101" s="89" t="n"/>
+      <c r="E101" s="89" t="n"/>
+      <c r="F101" s="89" t="n"/>
+      <c r="G101" s="89" t="n"/>
+      <c r="H101" s="89" t="n"/>
+      <c r="I101" s="89" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="89" t="n"/>
+      <c r="B102" s="89" t="n"/>
+      <c r="C102" s="89" t="n"/>
+      <c r="D102" s="89" t="n"/>
+      <c r="E102" s="89" t="n"/>
+      <c r="F102" s="89" t="n"/>
+      <c r="G102" s="89" t="n"/>
+      <c r="H102" s="89" t="n"/>
+      <c r="I102" s="89" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="89" t="n"/>
+      <c r="B103" s="89" t="n"/>
+      <c r="C103" s="89" t="n"/>
+      <c r="D103" s="89" t="n"/>
+      <c r="E103" s="89" t="n"/>
+      <c r="F103" s="89" t="n"/>
+      <c r="G103" s="89" t="n"/>
+      <c r="H103" s="89" t="n"/>
+      <c r="I103" s="89" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="A32:K32"/>
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="I5:I35">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"Hoàn thành"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3456,7 +4034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4523,9 +5101,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G40" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G40" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4558,9 +5136,9 @@
           <t>Khó</t>
         </is>
       </c>
-      <c r="G41" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G41" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4593,9 +5171,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G42" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G42" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4628,9 +5206,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G43" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G43" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4663,9 +5241,9 @@
           <t>Dễ</t>
         </is>
       </c>
-      <c r="G44" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G44" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4742,19 +5320,21 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G48" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G48" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
     <row r="49" ht="36" customHeight="1">
-      <c r="A49" s="79" t="n">
-        <v>2</v>
+      <c r="A49" s="79" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
       </c>
       <c r="B49" s="80" t="inlineStr">
         <is>
-          <t>Tùy Biến Thanh Tìm Kiếm Dạng Viên Thuốc (Pill Search)</t>
+          <t>Task 2.1: Tùy Biến Thanh Tìm Kiếm (Pill Search) &amp; Gỡ CSS Fix Kích Thước</t>
         </is>
       </c>
       <c r="C49" s="79" t="inlineStr">
@@ -4777,9 +5357,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G49" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G49" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4812,9 +5392,9 @@
           <t>Khó</t>
         </is>
       </c>
-      <c r="G50" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G50" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4847,9 +5427,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G51" s="83" t="inlineStr">
-        <is>
-          <t>Chờ thực hiện</t>
+      <c r="G51" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -4882,9 +5462,887 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="G52" s="83" t="inlineStr">
+      <c r="G52" s="85" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="96" t="inlineStr">
+        <is>
+          <t>VI. MA TRẬN BẺ KHỐI &amp; TỐI ƯU RESPONSIVE TRANG CHỦ (MOBILE &amp; TABLET)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="56" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B55" s="57" t="inlineStr">
+        <is>
+          <t>Tên Khối Giao Diện Cần Tối Ưu</t>
+        </is>
+      </c>
+      <c r="C55" s="56" t="inlineStr">
+        <is>
+          <t>Phân Loại Thành Phần</t>
+        </is>
+      </c>
+      <c r="D55" s="57" t="inlineStr">
+        <is>
+          <t>File / Template Can Thiệp</t>
+        </is>
+      </c>
+      <c r="E55" s="57" t="inlineStr">
+        <is>
+          <t>Phương Thức Triển Khai Kỹ Thuật</t>
+        </is>
+      </c>
+      <c r="F55" s="56" t="inlineStr">
+        <is>
+          <t>Độ Phức Tạp</t>
+        </is>
+      </c>
+      <c r="G55" s="56" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="36" customHeight="1">
+      <c r="A56" s="67" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B56" s="59" t="inlineStr">
+        <is>
+          <t>Chuyển Vị Trí Logo GoBike Sang Sát Lề Trái</t>
+        </is>
+      </c>
+      <c r="C56" s="58" t="inlineStr">
+        <is>
+          <t>Header Builder &amp; CSS</t>
+        </is>
+      </c>
+      <c r="D56" s="59" t="inlineStr">
+        <is>
+          <t>Flatsome Header Mobile &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E56" s="59" t="inlineStr">
+        <is>
+          <t>Yêu cầu từ ảnh: Chuyển vị trí Logo từ chính giữa sang bên trái nằm sát ngay sau Menu Icon; chỉnh max-height logo 46-48px vừa vặn</t>
+        </is>
+      </c>
+      <c r="F56" s="58" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G56" s="99" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="36" customHeight="1">
+      <c r="A57" s="67" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B57" s="59" t="inlineStr">
+        <is>
+          <t>Menu Hamburger 3 Gạch &amp; Off-Canvas Drawer</t>
+        </is>
+      </c>
+      <c r="C57" s="58" t="inlineStr">
+        <is>
+          <t>Mobile Nav &amp; Flatsome</t>
+        </is>
+      </c>
+      <c r="D57" s="59" t="inlineStr">
+        <is>
+          <t>Flatsome Header Mobile</t>
+        </is>
+      </c>
+      <c r="E57" s="59" t="inlineStr">
+        <is>
+          <t>Yêu cầu từ ảnh: Nút menu 3 gạch nền xanh lá (#00a651) bo góc vuông mềm; bấm mở trượt menu danh mục sản phẩm từ bên trái (off-canvas left)</t>
+        </is>
+      </c>
+      <c r="F57" s="58" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G57" s="99" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="36" customHeight="1">
+      <c r="A58" s="67" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B58" s="59" t="inlineStr">
+        <is>
+          <t>Cụm 2 Icon Tiện Ích Bên Phải Header</t>
+        </is>
+      </c>
+      <c r="C58" s="58" t="inlineStr">
+        <is>
+          <t>Header Icons &amp; CSS</t>
+        </is>
+      </c>
+      <c r="D58" s="59" t="inlineStr">
+        <is>
+          <t>Flatsome Header Mobile</t>
+        </is>
+      </c>
+      <c r="E58" s="59" t="inlineStr">
+        <is>
+          <t>Yêu cầu từ ảnh: Icon Định vị/Cửa hàng gần bạn (hình tròn xanh lá) + Icon Giỏ hàng (nền xanh lá bo góc) đặt sát lề phải</t>
+        </is>
+      </c>
+      <c r="F58" s="58" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G58" s="99" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="36" customHeight="1">
+      <c r="A59" s="67" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B59" s="59" t="inlineStr">
+        <is>
+          <t>Thanh Tìm Kiếm Viên Thuốc (Pill Search Mobile)</t>
+        </is>
+      </c>
+      <c r="C59" s="58" t="inlineStr">
+        <is>
+          <t>Search Element &amp; CSS</t>
+        </is>
+      </c>
+      <c r="D59" s="59" t="inlineStr">
+        <is>
+          <t>flatsome-child/style.css</t>
+        </is>
+      </c>
+      <c r="E59" s="59" t="inlineStr">
+        <is>
+          <t>Yêu cầu từ ảnh: Bố cục tầng 2 dạng viên thuốc bo tròn viền xám mờ; placeholder 'Bạn cần tìm gì?'; nút kính lúp tròn xanh lá ở góc phải</t>
+        </is>
+      </c>
+      <c r="F59" s="58" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G59" s="99" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="36" customHeight="1">
+      <c r="A60" s="67" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B60" s="59" t="inlineStr">
+        <is>
+          <t>Hero Section &amp; Slider Banner Mobile</t>
+        </is>
+      </c>
+      <c r="C60" s="58" t="inlineStr">
+        <is>
+          <t>UX Slider &amp; CSS</t>
+        </is>
+      </c>
+      <c r="D60" s="59" t="inlineStr">
+        <is>
+          <t>UX Builder &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E60" s="59" t="inlineStr">
+        <is>
+          <t>Co giãn chiều cao slider banner theo tỷ lệ màn hình điện thoại (touch swipe), chuyển khối tin tức nổi bật và banner 1H xuống dưới dạng carousel hoặc xếp chồng gọn</t>
+        </is>
+      </c>
+      <c r="F60" s="58" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G60" s="97" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1">
+      <c r="A61" s="67" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B61" s="59" t="inlineStr">
+        <is>
+          <t>Section Giờ Vàng Flash Sale Mobile</t>
+        </is>
+      </c>
+      <c r="C61" s="58" t="inlineStr">
+        <is>
+          <t>UX Tabs &amp; CSS Loop</t>
+        </is>
+      </c>
+      <c r="D61" s="59" t="inlineStr">
+        <is>
+          <t>UX Builder &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E61" s="59" t="inlineStr">
+        <is>
+          <t>Chuyển các tab khung giờ (17h, 19h, 20h, 21h) thành thanh cuộn ngang cảm ứng ngón tay (horizontal touch scroll), lưới sản phẩm sale co giãn 2 cột/dòng</t>
+        </is>
+      </c>
+      <c r="F61" s="58" t="inlineStr">
+        <is>
+          <t>Khó</t>
+        </is>
+      </c>
+      <c r="G61" s="97" t="inlineStr">
         <is>
           <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="36" customHeight="1">
+      <c r="A62" s="67" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B62" s="59" t="inlineStr">
+        <is>
+          <t>4 Khối Danh Mục Sản Phẩm (Shortcode 5 Cột)</t>
+        </is>
+      </c>
+      <c r="C62" s="58" t="inlineStr">
+        <is>
+          <t>PHP Shortcode &amp; CSS Grid</t>
+        </is>
+      </c>
+      <c r="D62" s="59" t="inlineStr">
+        <is>
+          <t>functions.php &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E62" s="59" t="inlineStr">
+        <is>
+          <t>Tối ưu shortcode [gobike_category_block]: Chuyển bố cục 1 Big Item 40% + 8 Small Items sang lưới 2 cột đều đặn trên mobile, ẩn bớt text dài tránh vỡ layout</t>
+        </is>
+      </c>
+      <c r="F62" s="58" t="inlineStr">
+        <is>
+          <t>Khó</t>
+        </is>
+      </c>
+      <c r="G62" s="97" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="36" customHeight="1">
+      <c r="A63" s="67" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B63" s="59" t="inlineStr">
+        <is>
+          <t>Tin Tức, Trust Badges &amp; Footer Mobile</t>
+        </is>
+      </c>
+      <c r="C63" s="58" t="inlineStr">
+        <is>
+          <t>CSS Media Queries &amp; QA</t>
+        </is>
+      </c>
+      <c r="D63" s="59" t="inlineStr">
+        <is>
+          <t>flatsome-child/style.css</t>
+        </is>
+      </c>
+      <c r="E63" s="59" t="inlineStr">
+        <is>
+          <t>Tin tức hiển thị dạng slider/1-2 cột, dải 4 cam kết cuộn ngang ngón tay, các cột footer xếp dọc 1 cột ngay ngắn, kiểm tra triệt để lỗi tràn ngang (overflow-x)</t>
+        </is>
+      </c>
+      <c r="F63" s="58" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G63" s="97" t="inlineStr">
+        <is>
+          <t>Chờ thực hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="96" t="inlineStr">
+        <is>
+          <t>VII. BẢNG TRA CỨU &amp; DANH MỤC SHORTCODE SỬ DỤNG CHO HEADER FLATSOME</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="28" customHeight="1">
+      <c r="A67" s="56" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B67" s="57" t="inlineStr">
+        <is>
+          <t>Tên Shortcode</t>
+        </is>
+      </c>
+      <c r="C67" s="57" t="inlineStr">
+        <is>
+          <t>Cú Pháp Chuẩn &amp; Tham Số (Syntax)</t>
+        </is>
+      </c>
+      <c r="D67" s="57" t="inlineStr">
+        <is>
+          <t>Vị Trí Áp Dụng Trên Header</t>
+        </is>
+      </c>
+      <c r="E67" s="57" t="inlineStr">
+        <is>
+          <t>Chức Năng &amp; Mục Đích Kỹ Thuật</t>
+        </is>
+      </c>
+      <c r="F67" s="56" t="inlineStr">
+        <is>
+          <t>Nguồn Gốc (Phân Loại)</t>
+        </is>
+      </c>
+      <c r="G67" s="56" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="36" customHeight="1">
+      <c r="A68" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="B68" s="100" t="inlineStr">
+        <is>
+          <t>Ticker Chạy Chữ Topbar</t>
+        </is>
+      </c>
+      <c r="C68" s="101" t="inlineStr">
+        <is>
+          <t>[gobike_topbar_ticker]</t>
+        </is>
+      </c>
+      <c r="D68" s="59" t="inlineStr">
+        <is>
+          <t>Top Bar (HTML 3 / Custom Text)</t>
+        </is>
+      </c>
+      <c r="E68" s="59" t="inlineStr">
+        <is>
+          <t>Chạy dòng chữ thông báo khuyến mãi, miễn phí giao hàng &amp; hotline trên thanh Top Bar</t>
+        </is>
+      </c>
+      <c r="F68" s="58" t="inlineStr">
+        <is>
+          <t>Custom Theme (functions.php)</t>
+        </is>
+      </c>
+      <c r="G68" s="60" t="inlineStr">
+        <is>
+          <t>Đang hoạt động</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="36" customHeight="1">
+      <c r="A69" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="B69" s="100" t="inlineStr">
+        <is>
+          <t>Thanh Tìm Kiếm Dạng Phẳng</t>
+        </is>
+      </c>
+      <c r="C69" s="101" t="inlineStr">
+        <is>
+          <t>[search style="flat"]</t>
+        </is>
+      </c>
+      <c r="D69" s="59" t="inlineStr">
+        <is>
+          <t>Header Main / Mobile (HTML 1 hoặc 5)</t>
+        </is>
+      </c>
+      <c r="E69" s="59" t="inlineStr">
+        <is>
+          <t>Hiển thị khung tìm kiếm phẳng, bo cong góc, tích hợp AJAX live search sản phẩm tức thì</t>
+        </is>
+      </c>
+      <c r="F69" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Core Shortcode</t>
+        </is>
+      </c>
+      <c r="G69" s="60" t="inlineStr">
+        <is>
+          <t>Đang áp dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="36" customHeight="1">
+      <c r="A70" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="B70" s="100" t="inlineStr">
+        <is>
+          <t>Thanh Tìm Kiếm Tiêu Chuẩn</t>
+        </is>
+      </c>
+      <c r="C70" s="101" t="inlineStr">
+        <is>
+          <t>[search style="normal" size="small"]</t>
+        </is>
+      </c>
+      <c r="D70" s="59" t="inlineStr">
+        <is>
+          <t>Header Bottom / Header Sticky</t>
+        </is>
+      </c>
+      <c r="E70" s="59" t="inlineStr">
+        <is>
+          <t>Thanh tìm kiếm viền nét bo tròn có nút bấm kính lúp độc lập, hỗ trợ tùy chỉnh kích cỡ</t>
+        </is>
+      </c>
+      <c r="F70" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Core Shortcode</t>
+        </is>
+      </c>
+      <c r="G70" s="99" t="inlineStr">
+        <is>
+          <t>Sẵn sàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="36" customHeight="1">
+      <c r="A71" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="B71" s="100" t="inlineStr">
+        <is>
+          <t>Nhúng Khối UX Block / Mega Menu</t>
+        </is>
+      </c>
+      <c r="C71" s="101" t="inlineStr">
+        <is>
+          <t>[block id="slug-ux-block"]</t>
+        </is>
+      </c>
+      <c r="D71" s="59" t="inlineStr">
+        <is>
+          <t>Mega Menu Dropdown / Header Bottom</t>
+        </is>
+      </c>
+      <c r="E71" s="59" t="inlineStr">
+        <is>
+          <t>Nhúng bất kỳ khối thiết kế UX Builder tùy biến nào vào menu đa tầng hoặc chân header</t>
+        </is>
+      </c>
+      <c r="F71" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Core Shortcode</t>
+        </is>
+      </c>
+      <c r="G71" s="60" t="inlineStr">
+        <is>
+          <t>Đang áp dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="36" customHeight="1">
+      <c r="A72" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="B72" s="100" t="inlineStr">
+        <is>
+          <t>Nút Bấm Tiện Ích Bo Tròn</t>
+        </is>
+      </c>
+      <c r="C72" s="101" t="inlineStr">
+        <is>
+          <t>[button text="Hotline" link="tel:..." style="primary" radius="99px" icon="icon-phone"]</t>
+        </is>
+      </c>
+      <c r="D72" s="59" t="inlineStr">
+        <is>
+          <t>Header Right (HTML / Button)</t>
+        </is>
+      </c>
+      <c r="E72" s="59" t="inlineStr">
+        <is>
+          <t>Tạo nút Hotline hoặc Cửa hàng gần bạn bo tròn viên thuốc kèm icon nhận diện GoBike</t>
+        </is>
+      </c>
+      <c r="F72" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Core Shortcode</t>
+        </is>
+      </c>
+      <c r="G72" s="60" t="inlineStr">
+        <is>
+          <t>Đang áp dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="36" customHeight="1">
+      <c r="A73" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="B73" s="100" t="inlineStr">
+        <is>
+          <t>Chuỗi Icon Mạng Xã Hội</t>
+        </is>
+      </c>
+      <c r="C73" s="101" t="inlineStr">
+        <is>
+          <t>[follow facebook="url" tiktok="url" youtube="url"]</t>
+        </is>
+      </c>
+      <c r="D73" s="59" t="inlineStr">
+        <is>
+          <t>Top Bar / Menu Trượt Off-Canvas</t>
+        </is>
+      </c>
+      <c r="E73" s="59" t="inlineStr">
+        <is>
+          <t>Hiển thị chuỗi icon liên kết mạng xã hội chính thức (Facebook, TikTok, YouTube) bo tròn</t>
+        </is>
+      </c>
+      <c r="F73" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Core Shortcode</t>
+        </is>
+      </c>
+      <c r="G73" s="99" t="inlineStr">
+        <is>
+          <t>Sẵn sàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="36" customHeight="1">
+      <c r="A74" s="67" t="n">
+        <v>7</v>
+      </c>
+      <c r="B74" s="100" t="inlineStr">
+        <is>
+          <t>Menu Điều Hướng Nhúng</t>
+        </is>
+      </c>
+      <c r="C74" s="101" t="inlineStr">
+        <is>
+          <t>[ux_menu id="slug-menu"]</t>
+        </is>
+      </c>
+      <c r="D74" s="59" t="inlineStr">
+        <is>
+          <t>Header Mobile / Off-Canvas Drawer</t>
+        </is>
+      </c>
+      <c r="E74" s="59" t="inlineStr">
+        <is>
+          <t>Nhúng một menu WordPress đã tạo sẵn vào bất kỳ vị trí HTML nào trên thanh Header</t>
+        </is>
+      </c>
+      <c r="F74" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Core Shortcode</t>
+        </is>
+      </c>
+      <c r="G74" s="99" t="inlineStr">
+        <is>
+          <t>Sẵn sàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="36" customHeight="1">
+      <c r="A75" s="67" t="n">
+        <v>8</v>
+      </c>
+      <c r="B75" s="100" t="inlineStr">
+        <is>
+          <t>Ảnh Logo Tùy Biến Mobile</t>
+        </is>
+      </c>
+      <c r="C75" s="101" t="inlineStr">
+        <is>
+          <t>[ux_image id="img_id" width="120px"]</t>
+        </is>
+      </c>
+      <c r="D75" s="59" t="inlineStr">
+        <is>
+          <t>Header Left Mobile (Khối HTML)</t>
+        </is>
+      </c>
+      <c r="E75" s="59" t="inlineStr">
+        <is>
+          <t>Chèn logo độc lập cho Mobile khi muốn tách biệt vị trí với Logo Desktop mà không bị khóa</t>
+        </is>
+      </c>
+      <c r="F75" s="58" t="inlineStr">
+        <is>
+          <t>Flatsome Core Shortcode</t>
+        </is>
+      </c>
+      <c r="G75" s="99" t="inlineStr">
+        <is>
+          <t>Sẵn sàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="96" t="inlineStr">
+        <is>
+          <t>VIII. MA TRẬN BẺ KHỐI &amp; KỸ THUẬT XÂY DỰNG MOBILE BOTTOM NAVIGATION BAR (THEO THIẾT KẾ MẪU ẢNH 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="56" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B78" s="56" t="inlineStr">
+        <is>
+          <t>Tên Khối Giao Diện / Tính Năng</t>
+        </is>
+      </c>
+      <c r="C78" s="56" t="inlineStr">
+        <is>
+          <t>Phân Loại Thành Phần</t>
+        </is>
+      </c>
+      <c r="D78" s="56" t="inlineStr">
+        <is>
+          <t>File / Template Can Thiệp</t>
+        </is>
+      </c>
+      <c r="E78" s="56" t="inlineStr">
+        <is>
+          <t>Phương Thức Triển Khai Kỹ Thuật</t>
+        </is>
+      </c>
+      <c r="F78" s="56" t="inlineStr">
+        <is>
+          <t>Độ Phức Tạp</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="B79" s="105" t="inlineStr">
+        <is>
+          <t>Khởi Tạo Khung Thanh Menu Dính Đáy Mobile</t>
+        </is>
+      </c>
+      <c r="C79" s="58" t="inlineStr">
+        <is>
+          <t>Custom Footer HTML &amp; Hook</t>
+        </is>
+      </c>
+      <c r="D79" s="104" t="inlineStr">
+        <is>
+          <t>flatsome-child/functions.php</t>
+        </is>
+      </c>
+      <c r="E79" s="59" t="inlineStr">
+        <is>
+          <t>Móc vào hook wp_footer tạo khung cố định chân trang (#gobike-bottom-nav), áp dụng position: fixed; bottom: 0; left: 0; width: 100%; z-index: 999; flexbox chia đều 5 cột</t>
+        </is>
+      </c>
+      <c r="F79" s="58" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="B80" s="105" t="inlineStr">
+        <is>
+          <t>Xây Dựng 4 Nút Tiện Ích Phẳng 2 Bên (Trang chủ, Sản phẩm, Messenger, Zalo)</t>
+        </is>
+      </c>
+      <c r="C80" s="58" t="inlineStr">
+        <is>
+          <t>Icon Box &amp; Action Links</t>
+        </is>
+      </c>
+      <c r="D80" s="104" t="inlineStr">
+        <is>
+          <t>functions.php &amp; style.css</t>
+        </is>
+      </c>
+      <c r="E80" s="59" t="inlineStr">
+        <is>
+          <t>Thiết kế 4 nút điều hướng phẳng gồm Icon SVG/FontAwesome bên trên + Label chữ nhỏ bên dưới; gắn link Trang chủ (/), Danh mục Sản phẩm (/san-pham/), link chat Zalo (zalo.me) &amp; Messenger (m.me)</t>
+        </is>
+      </c>
+      <c r="F80" s="58" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="B81" s="105" t="inlineStr">
+        <is>
+          <t>Thiết Kế Nút Gọi Điện Tròn Nổi Bật (Raised Center FAB)</t>
+        </is>
+      </c>
+      <c r="C81" s="58" t="inlineStr">
+        <is>
+          <t>Floating Button &amp; Animation</t>
+        </is>
+      </c>
+      <c r="D81" s="104" t="inlineStr">
+        <is>
+          <t>flatsome-child/style.css</t>
+        </is>
+      </c>
+      <c r="E81" s="59" t="inlineStr">
+        <is>
+          <t>Nút hotline ở vị trí trung tâm (nút thứ 3): Bo tròn 52px, nền đỏ #d0021b, viền trắng 3px, nhô cao lên trên thanh bar (transform: translateY(-18px)), đổ bóng 3D nổi bật kèm hiệu ứng pulse sóng rung thu hút khách gọi</t>
+        </is>
+      </c>
+      <c r="F81" s="58" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="B82" s="105" t="inlineStr">
+        <is>
+          <t>Media Queries &amp; Khoảng Đệm An Toàn (Safe Area)</t>
+        </is>
+      </c>
+      <c r="C82" s="58" t="inlineStr">
+        <is>
+          <t>CSS Responsive &amp; Safe-area</t>
+        </is>
+      </c>
+      <c r="D82" s="104" t="inlineStr">
+        <is>
+          <t>flatsome-child/style.css</t>
+        </is>
+      </c>
+      <c r="E82" s="59" t="inlineStr">
+        <is>
+          <t>Chỉ hiển thị trên màn hình Mobile/Tablet (@media max-width: 849px), ẩn hoàn toàn trên Desktop. Thêm padding-bottom 65-70px cho body/footer trên mobile để thanh cố định không che khuất nội dung website</t>
+        </is>
+      </c>
+      <c r="F82" s="58" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="B83" s="105" t="inlineStr">
+        <is>
+          <t>Kiểm Thử Trải Nghiệm Touch &amp; Tối Ưu Tương Thích iOS/Android</t>
+        </is>
+      </c>
+      <c r="C83" s="58" t="inlineStr">
+        <is>
+          <t>QA Mobile Testing &amp; CSS</t>
+        </is>
+      </c>
+      <c r="D83" s="104" t="inlineStr">
+        <is>
+          <t>flatsome-child/style.css</t>
+        </is>
+      </c>
+      <c r="E83" s="59" t="inlineStr">
+        <is>
+          <t>Hỗ trợ dải an toàn iPhone (env(safe-area-inset-bottom)), kiểm thử cảm ứng bấm mượt mà, phản hồi tap nhanh chóng, không bị lag hay xung đột với thanh header sticky</t>
+        </is>
+      </c>
+      <c r="F83" s="58" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>100% Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>